<commit_message>
money excel style finish
</commit_message>
<xml_diff>
--- a/output/2026/money.xlsx
+++ b/output/2026/money.xlsx
@@ -84,7 +84,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -144,11 +144,131 @@
       <bottom style="medium"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="dashed"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="dashed"/>
+      <top style="medium"/>
+      <bottom style="dashed"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="dashed"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="dashed"/>
+      <top style="medium"/>
+      <bottom style="dashed"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="dashed"/>
+      <bottom style="dashed"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="dashed"/>
+      <top style="dashed"/>
+      <bottom style="dashed"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="medium"/>
+      <top style="dashed"/>
+      <bottom style="dashed"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="dashed"/>
+      <top style="dashed"/>
+      <bottom style="dashed"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="dashed"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="dashed"/>
+      <top style="dashed"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="medium"/>
+      <top style="dashed"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="dashed"/>
+      <top style="dashed"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="dashed"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="dashed"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="dashed"/>
+      <top style="thin"/>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="medium"/>
+    </border>
+    <border>
+      <left style="dashed"/>
+      <right style="dashed"/>
+      <top style="thin"/>
+      <bottom style="medium"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -206,7 +326,131 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -588,25 +832,25 @@
   <dimension ref="A2:T38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10.5" customWidth="1" min="3" max="3"/>
-    <col width="10.5" customWidth="1" min="4" max="4"/>
-    <col width="10.5" customWidth="1" min="5" max="5"/>
-    <col width="10.5" customWidth="1" min="6" max="6"/>
-    <col width="10.5" customWidth="1" min="7" max="7"/>
-    <col width="10.5" customWidth="1" min="8" max="8"/>
-    <col width="10.5" customWidth="1" min="9" max="9"/>
-    <col width="10.5" customWidth="1" min="10" max="10"/>
-    <col width="10.5" customWidth="1" min="11" max="11"/>
-    <col width="10.5" customWidth="1" min="12" max="12"/>
-    <col width="10.5" customWidth="1" min="13" max="13"/>
-    <col width="10.5" customWidth="1" min="14" max="14"/>
-    <col width="10.5" customWidth="1" min="15" max="15"/>
-    <col width="10.5" customWidth="1" min="16" max="16"/>
-    <col width="10.5" customWidth="1" min="17" max="17"/>
-    <col width="10.5" customWidth="1" min="18" max="18"/>
-    <col width="10.5" customWidth="1" min="19" max="19"/>
-    <col width="10.5" customWidth="1" min="20" max="20"/>
+    <col width="14.5" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -814,402 +1058,587 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="G5" s="41" t="inlineStr">
+      <c r="C5" s="42" t="n"/>
+      <c r="D5" s="43" t="n"/>
+      <c r="E5" s="44" t="n"/>
+      <c r="F5" s="45" t="n"/>
+      <c r="G5" s="46" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="H5" s="41" t="inlineStr">
+      <c r="H5" s="47" t="inlineStr">
         <is>
           <t>14.6</t>
         </is>
       </c>
-      <c r="O5" s="41" t="inlineStr">
+      <c r="I5" s="48" t="n"/>
+      <c r="J5" s="49" t="n"/>
+      <c r="K5" s="50" t="n"/>
+      <c r="L5" s="51" t="n"/>
+      <c r="M5" s="52" t="n"/>
+      <c r="N5" s="53" t="n"/>
+      <c r="O5" s="54" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="P5" s="41" t="inlineStr">
+      <c r="P5" s="55" t="inlineStr">
         <is>
           <t>14.6</t>
         </is>
       </c>
-      <c r="Q5" s="41" t="inlineStr">
+      <c r="Q5" s="56" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="R5" s="41" t="inlineStr">
+      <c r="R5" s="57" t="inlineStr">
         <is>
           <t>14.6</t>
         </is>
       </c>
+      <c r="S5" s="58" t="n"/>
+      <c r="T5" s="59" t="n"/>
     </row>
     <row r="6">
-      <c r="G6" s="41" t="inlineStr">
+      <c r="B6" s="60" t="n"/>
+      <c r="C6" s="61" t="n"/>
+      <c r="D6" s="62" t="n"/>
+      <c r="E6" s="63" t="n"/>
+      <c r="F6" s="64" t="n"/>
+      <c r="G6" s="65" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="H6" s="41" t="inlineStr">
+      <c r="H6" s="66" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="O6" s="41" t="inlineStr">
+      <c r="I6" s="67" t="n"/>
+      <c r="J6" s="68" t="n"/>
+      <c r="K6" s="69" t="n"/>
+      <c r="L6" s="70" t="n"/>
+      <c r="M6" s="71" t="n"/>
+      <c r="N6" s="72" t="n"/>
+      <c r="O6" s="73" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="P6" s="41" t="inlineStr">
+      <c r="P6" s="74" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="Q6" s="41" t="inlineStr">
+      <c r="Q6" s="75" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="R6" s="41" t="inlineStr">
+      <c r="R6" s="76" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
+      <c r="S6" s="77" t="n"/>
+      <c r="T6" s="78" t="n"/>
     </row>
     <row r="7">
-      <c r="E7" s="41" t="inlineStr">
+      <c r="B7" s="60" t="n"/>
+      <c r="C7" s="61" t="n"/>
+      <c r="D7" s="62" t="n"/>
+      <c r="E7" s="79" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F7" s="41" t="inlineStr">
+      <c r="F7" s="80" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="I7" s="41" t="inlineStr">
+      <c r="G7" s="81" t="n"/>
+      <c r="H7" s="82" t="n"/>
+      <c r="I7" s="83" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="J7" s="41" t="inlineStr">
+      <c r="J7" s="84" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="K7" s="69" t="n"/>
+      <c r="L7" s="70" t="n"/>
+      <c r="M7" s="71" t="n"/>
+      <c r="N7" s="72" t="n"/>
+      <c r="O7" s="85" t="n"/>
+      <c r="P7" s="86" t="n"/>
+      <c r="Q7" s="87" t="n"/>
+      <c r="R7" s="88" t="n"/>
+      <c r="S7" s="77" t="n"/>
+      <c r="T7" s="78" t="n"/>
     </row>
     <row r="8">
-      <c r="I8" s="41" t="inlineStr">
+      <c r="B8" s="60" t="n"/>
+      <c r="C8" s="61" t="n"/>
+      <c r="D8" s="62" t="n"/>
+      <c r="E8" s="63" t="n"/>
+      <c r="F8" s="64" t="n"/>
+      <c r="G8" s="81" t="n"/>
+      <c r="H8" s="82" t="n"/>
+      <c r="I8" s="83" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="J8" s="41" t="inlineStr">
+      <c r="J8" s="84" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="O8" s="41" t="inlineStr">
+      <c r="K8" s="69" t="n"/>
+      <c r="L8" s="70" t="n"/>
+      <c r="M8" s="71" t="n"/>
+      <c r="N8" s="72" t="n"/>
+      <c r="O8" s="73" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="P8" s="41" t="inlineStr">
+      <c r="P8" s="74" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="Q8" s="41" t="inlineStr">
+      <c r="Q8" s="75" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="R8" s="41" t="inlineStr">
+      <c r="R8" s="76" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
+      <c r="S8" s="77" t="n"/>
+      <c r="T8" s="78" t="n"/>
     </row>
     <row r="9">
-      <c r="E9" s="41" t="inlineStr">
+      <c r="B9" s="60" t="n"/>
+      <c r="C9" s="61" t="n"/>
+      <c r="D9" s="62" t="n"/>
+      <c r="E9" s="79" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F9" s="41" t="inlineStr">
+      <c r="F9" s="80" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
-      <c r="I9" s="41" t="inlineStr">
+      <c r="G9" s="81" t="n"/>
+      <c r="H9" s="82" t="n"/>
+      <c r="I9" s="83" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
-      <c r="J9" s="41" t="inlineStr">
+      <c r="J9" s="84" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="K9" s="69" t="n"/>
+      <c r="L9" s="70" t="n"/>
+      <c r="M9" s="71" t="n"/>
+      <c r="N9" s="72" t="n"/>
+      <c r="O9" s="85" t="n"/>
+      <c r="P9" s="86" t="n"/>
+      <c r="Q9" s="87" t="n"/>
+      <c r="R9" s="88" t="n"/>
+      <c r="S9" s="77" t="n"/>
+      <c r="T9" s="78" t="n"/>
     </row>
     <row r="10">
-      <c r="I10" s="41" t="inlineStr">
+      <c r="B10" s="60" t="n"/>
+      <c r="C10" s="61" t="n"/>
+      <c r="D10" s="62" t="n"/>
+      <c r="E10" s="63" t="n"/>
+      <c r="F10" s="64" t="n"/>
+      <c r="G10" s="81" t="n"/>
+      <c r="H10" s="82" t="n"/>
+      <c r="I10" s="83" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="J10" s="41" t="inlineStr">
+      <c r="J10" s="84" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
-      <c r="O10" s="41" t="inlineStr">
+      <c r="K10" s="69" t="n"/>
+      <c r="L10" s="70" t="n"/>
+      <c r="M10" s="71" t="n"/>
+      <c r="N10" s="72" t="n"/>
+      <c r="O10" s="73" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="P10" s="41" t="inlineStr">
+      <c r="P10" s="74" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
-      <c r="Q10" s="41" t="inlineStr">
+      <c r="Q10" s="75" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="R10" s="41" t="inlineStr">
+      <c r="R10" s="76" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
+      <c r="S10" s="77" t="n"/>
+      <c r="T10" s="78" t="n"/>
     </row>
     <row r="11">
-      <c r="E11" s="41" t="inlineStr">
+      <c r="B11" s="60" t="n"/>
+      <c r="C11" s="61" t="n"/>
+      <c r="D11" s="62" t="n"/>
+      <c r="E11" s="79" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F11" s="41" t="inlineStr">
+      <c r="F11" s="80" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="M11" s="41" t="inlineStr">
+      <c r="G11" s="81" t="n"/>
+      <c r="H11" s="82" t="n"/>
+      <c r="I11" s="67" t="n"/>
+      <c r="J11" s="68" t="n"/>
+      <c r="K11" s="69" t="n"/>
+      <c r="L11" s="70" t="n"/>
+      <c r="M11" s="89" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="N11" s="41" t="inlineStr">
+      <c r="N11" s="90" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="O11" s="85" t="n"/>
+      <c r="P11" s="86" t="n"/>
+      <c r="Q11" s="87" t="n"/>
+      <c r="R11" s="88" t="n"/>
+      <c r="S11" s="77" t="n"/>
+      <c r="T11" s="78" t="n"/>
     </row>
     <row r="12">
-      <c r="M12" s="41" t="inlineStr">
+      <c r="B12" s="60" t="n"/>
+      <c r="C12" s="61" t="n"/>
+      <c r="D12" s="62" t="n"/>
+      <c r="E12" s="63" t="n"/>
+      <c r="F12" s="64" t="n"/>
+      <c r="G12" s="81" t="n"/>
+      <c r="H12" s="82" t="n"/>
+      <c r="I12" s="67" t="n"/>
+      <c r="J12" s="68" t="n"/>
+      <c r="K12" s="69" t="n"/>
+      <c r="L12" s="70" t="n"/>
+      <c r="M12" s="89" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="N12" s="41" t="inlineStr">
+      <c r="N12" s="90" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="O12" s="41" t="inlineStr">
+      <c r="O12" s="73" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="P12" s="41" t="inlineStr">
+      <c r="P12" s="74" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="Q12" s="41" t="inlineStr">
+      <c r="Q12" s="75" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="R12" s="41" t="inlineStr">
+      <c r="R12" s="76" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
+      <c r="S12" s="77" t="n"/>
+      <c r="T12" s="78" t="n"/>
     </row>
     <row r="13">
-      <c r="E13" s="41" t="inlineStr">
+      <c r="B13" s="60" t="n"/>
+      <c r="C13" s="61" t="n"/>
+      <c r="D13" s="62" t="n"/>
+      <c r="E13" s="79" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F13" s="41" t="inlineStr">
+      <c r="F13" s="80" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
-      <c r="I13" s="41" t="inlineStr">
+      <c r="G13" s="81" t="n"/>
+      <c r="H13" s="82" t="n"/>
+      <c r="I13" s="83" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
-      <c r="J13" s="41" t="inlineStr">
+      <c r="J13" s="84" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="K13" s="69" t="n"/>
+      <c r="L13" s="70" t="n"/>
+      <c r="M13" s="71" t="n"/>
+      <c r="N13" s="72" t="n"/>
+      <c r="O13" s="85" t="n"/>
+      <c r="P13" s="86" t="n"/>
+      <c r="Q13" s="87" t="n"/>
+      <c r="R13" s="88" t="n"/>
+      <c r="S13" s="77" t="n"/>
+      <c r="T13" s="78" t="n"/>
     </row>
     <row r="14">
-      <c r="I14" s="41" t="inlineStr">
+      <c r="B14" s="60" t="n"/>
+      <c r="C14" s="61" t="n"/>
+      <c r="D14" s="62" t="n"/>
+      <c r="E14" s="63" t="n"/>
+      <c r="F14" s="64" t="n"/>
+      <c r="G14" s="81" t="n"/>
+      <c r="H14" s="82" t="n"/>
+      <c r="I14" s="83" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="J14" s="41" t="inlineStr">
+      <c r="J14" s="84" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
-      <c r="O14" s="41" t="inlineStr">
+      <c r="K14" s="69" t="n"/>
+      <c r="L14" s="70" t="n"/>
+      <c r="M14" s="71" t="n"/>
+      <c r="N14" s="72" t="n"/>
+      <c r="O14" s="73" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="P14" s="41" t="inlineStr">
+      <c r="P14" s="74" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
-      <c r="Q14" s="41" t="inlineStr">
+      <c r="Q14" s="75" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="R14" s="41" t="inlineStr">
+      <c r="R14" s="76" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
+      <c r="S14" s="77" t="n"/>
+      <c r="T14" s="78" t="n"/>
     </row>
     <row r="15">
-      <c r="E15" s="41" t="inlineStr">
+      <c r="B15" s="60" t="n"/>
+      <c r="C15" s="61" t="n"/>
+      <c r="D15" s="62" t="n"/>
+      <c r="E15" s="79" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F15" s="41" t="inlineStr">
+      <c r="F15" s="80" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
-      <c r="I15" s="41" t="inlineStr">
+      <c r="G15" s="81" t="n"/>
+      <c r="H15" s="82" t="n"/>
+      <c r="I15" s="83" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
-      <c r="J15" s="41" t="inlineStr">
+      <c r="J15" s="84" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="K15" s="69" t="n"/>
+      <c r="L15" s="70" t="n"/>
+      <c r="M15" s="71" t="n"/>
+      <c r="N15" s="72" t="n"/>
+      <c r="O15" s="85" t="n"/>
+      <c r="P15" s="86" t="n"/>
+      <c r="Q15" s="87" t="n"/>
+      <c r="R15" s="88" t="n"/>
+      <c r="S15" s="77" t="n"/>
+      <c r="T15" s="78" t="n"/>
     </row>
     <row r="16">
-      <c r="I16" s="41" t="inlineStr">
+      <c r="B16" s="91" t="n"/>
+      <c r="C16" s="92" t="n"/>
+      <c r="D16" s="93" t="n"/>
+      <c r="E16" s="94" t="n"/>
+      <c r="F16" s="95" t="n"/>
+      <c r="G16" s="96" t="n"/>
+      <c r="H16" s="97" t="n"/>
+      <c r="I16" s="98" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="J16" s="41" t="inlineStr">
+      <c r="J16" s="99" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
-      <c r="O16" s="41" t="inlineStr">
+      <c r="K16" s="100" t="n"/>
+      <c r="L16" s="101" t="n"/>
+      <c r="M16" s="102" t="n"/>
+      <c r="N16" s="103" t="n"/>
+      <c r="O16" s="104" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="P16" s="41" t="inlineStr">
+      <c r="P16" s="105" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
-      <c r="Q16" s="41" t="inlineStr">
+      <c r="Q16" s="106" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="R16" s="41" t="inlineStr">
+      <c r="R16" s="107" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
+      <c r="S16" s="108" t="n"/>
+      <c r="T16" s="109" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="41" t="inlineStr">
+      <c r="B17" s="110" t="inlineStr">
         <is>
           <t>sum</t>
         </is>
       </c>
-      <c r="C17" s="41" t="n">
+      <c r="C17" s="111" t="n">
         <v>70</v>
       </c>
-      <c r="E17" s="41" t="n">
+      <c r="D17" s="112" t="n"/>
+      <c r="E17" s="113" t="n">
         <v>14944.22</v>
       </c>
-      <c r="G17" s="41" t="n">
+      <c r="F17" s="114" t="n"/>
+      <c r="G17" s="115" t="n">
         <v>68</v>
       </c>
-      <c r="I17" s="41" t="n">
+      <c r="H17" s="116" t="n"/>
+      <c r="I17" s="117" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="41" t="n">
+      <c r="J17" s="118" t="n"/>
+      <c r="K17" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="M17" s="41" t="n">
+      <c r="L17" s="120" t="n"/>
+      <c r="M17" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="O17" s="41" t="n">
+      <c r="N17" s="122" t="n"/>
+      <c r="O17" s="123" t="n">
         <v>0</v>
       </c>
-      <c r="P17" s="41" t="n">
+      <c r="P17" s="124" t="n">
         <v>343.7</v>
       </c>
-      <c r="Q17" s="41" t="n">
+      <c r="Q17" s="125" t="n">
         <v>0</v>
       </c>
-      <c r="R17" s="41" t="n">
+      <c r="R17" s="126" t="n">
         <v>343.7</v>
       </c>
-      <c r="S17" s="41" t="n">
+      <c r="S17" s="127" t="n">
         <v>15082.22</v>
       </c>
-      <c r="T17" s="41" t="inlineStr">
+      <c r="T17" s="128" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="41" t="inlineStr">
+      <c r="B18" s="129" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="O18" s="41" t="n">
+      <c r="C18" s="130" t="n"/>
+      <c r="D18" s="131" t="n"/>
+      <c r="E18" s="132" t="n"/>
+      <c r="F18" s="133" t="n"/>
+      <c r="G18" s="134" t="n"/>
+      <c r="H18" s="135" t="n"/>
+      <c r="I18" s="136" t="n"/>
+      <c r="J18" s="137" t="n"/>
+      <c r="K18" s="138" t="n"/>
+      <c r="L18" s="139" t="n"/>
+      <c r="M18" s="140" t="n"/>
+      <c r="N18" s="141" t="n"/>
+      <c r="O18" s="142" t="n">
         <v>0</v>
       </c>
-      <c r="P18" s="41" t="n">
+      <c r="P18" s="143" t="n">
         <v>343.7</v>
       </c>
-      <c r="Q18" s="41" t="n">
+      <c r="Q18" s="144" t="n">
         <v>0</v>
       </c>
-      <c r="R18" s="41" t="n">
+      <c r="R18" s="145" t="n">
         <v>343.7</v>
       </c>
+      <c r="S18" s="146" t="n"/>
+      <c r="T18" s="147" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="41" t="inlineStr">
@@ -1217,600 +1646,859 @@
           <t>02/01/2026</t>
         </is>
       </c>
-      <c r="E19" s="41" t="inlineStr">
+      <c r="C19" s="42" t="n"/>
+      <c r="D19" s="43" t="n"/>
+      <c r="E19" s="148" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
-      <c r="F19" s="41" t="inlineStr">
+      <c r="F19" s="149" t="inlineStr">
         <is>
           <t>2993</t>
         </is>
       </c>
-      <c r="Q19" s="41" t="inlineStr">
+      <c r="G19" s="150" t="n"/>
+      <c r="H19" s="151" t="n"/>
+      <c r="I19" s="48" t="n"/>
+      <c r="J19" s="49" t="n"/>
+      <c r="K19" s="50" t="n"/>
+      <c r="L19" s="51" t="n"/>
+      <c r="M19" s="52" t="n"/>
+      <c r="N19" s="53" t="n"/>
+      <c r="O19" s="152" t="n"/>
+      <c r="P19" s="153" t="n"/>
+      <c r="Q19" s="56" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
-      <c r="R19" s="41" t="inlineStr">
+      <c r="R19" s="57" t="inlineStr">
         <is>
           <t>2993</t>
         </is>
       </c>
+      <c r="S19" s="58" t="n"/>
+      <c r="T19" s="59" t="n"/>
     </row>
     <row r="20">
-      <c r="E20" s="41" t="inlineStr">
+      <c r="B20" s="60" t="n"/>
+      <c r="C20" s="61" t="n"/>
+      <c r="D20" s="62" t="n"/>
+      <c r="E20" s="79" t="inlineStr">
         <is>
           <t>7000</t>
         </is>
       </c>
-      <c r="F20" s="41" t="inlineStr">
+      <c r="F20" s="80" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
-      <c r="Q20" s="41" t="inlineStr">
+      <c r="G20" s="81" t="n"/>
+      <c r="H20" s="82" t="n"/>
+      <c r="I20" s="67" t="n"/>
+      <c r="J20" s="68" t="n"/>
+      <c r="K20" s="69" t="n"/>
+      <c r="L20" s="70" t="n"/>
+      <c r="M20" s="71" t="n"/>
+      <c r="N20" s="72" t="n"/>
+      <c r="O20" s="85" t="n"/>
+      <c r="P20" s="86" t="n"/>
+      <c r="Q20" s="75" t="inlineStr">
         <is>
           <t>7000</t>
         </is>
       </c>
-      <c r="R20" s="41" t="inlineStr">
+      <c r="R20" s="76" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
+      <c r="S20" s="77" t="n"/>
+      <c r="T20" s="78" t="n"/>
     </row>
     <row r="21">
-      <c r="G21" s="41" t="inlineStr">
+      <c r="B21" s="60" t="n"/>
+      <c r="C21" s="61" t="n"/>
+      <c r="D21" s="62" t="n"/>
+      <c r="E21" s="63" t="n"/>
+      <c r="F21" s="64" t="n"/>
+      <c r="G21" s="65" t="inlineStr">
         <is>
           <t>LRT</t>
         </is>
       </c>
-      <c r="H21" s="41" t="inlineStr">
+      <c r="H21" s="66" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="O21" s="41" t="inlineStr">
+      <c r="I21" s="67" t="n"/>
+      <c r="J21" s="68" t="n"/>
+      <c r="K21" s="69" t="n"/>
+      <c r="L21" s="70" t="n"/>
+      <c r="M21" s="71" t="n"/>
+      <c r="N21" s="72" t="n"/>
+      <c r="O21" s="73" t="inlineStr">
         <is>
           <t>LRT</t>
         </is>
       </c>
-      <c r="P21" s="41" t="inlineStr">
+      <c r="P21" s="74" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="Q21" s="41" t="inlineStr">
+      <c r="Q21" s="75" t="inlineStr">
         <is>
           <t>LRT</t>
         </is>
       </c>
-      <c r="R21" s="41" t="inlineStr">
+      <c r="R21" s="76" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
+      <c r="S21" s="77" t="n"/>
+      <c r="T21" s="78" t="n"/>
     </row>
     <row r="22">
-      <c r="G22" s="41" t="inlineStr">
+      <c r="B22" s="60" t="n"/>
+      <c r="C22" s="61" t="n"/>
+      <c r="D22" s="62" t="n"/>
+      <c r="E22" s="63" t="n"/>
+      <c r="F22" s="64" t="n"/>
+      <c r="G22" s="65" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="H22" s="41" t="inlineStr">
+      <c r="H22" s="66" t="inlineStr">
         <is>
           <t>10.8</t>
         </is>
       </c>
-      <c r="O22" s="41" t="inlineStr">
+      <c r="I22" s="67" t="n"/>
+      <c r="J22" s="68" t="n"/>
+      <c r="K22" s="69" t="n"/>
+      <c r="L22" s="70" t="n"/>
+      <c r="M22" s="71" t="n"/>
+      <c r="N22" s="72" t="n"/>
+      <c r="O22" s="73" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="P22" s="41" t="inlineStr">
+      <c r="P22" s="74" t="inlineStr">
         <is>
           <t>10.8</t>
         </is>
       </c>
-      <c r="Q22" s="41" t="inlineStr">
+      <c r="Q22" s="75" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="R22" s="41" t="inlineStr">
+      <c r="R22" s="76" t="inlineStr">
         <is>
           <t>10.8</t>
         </is>
       </c>
+      <c r="S22" s="77" t="n"/>
+      <c r="T22" s="78" t="n"/>
     </row>
     <row r="23">
-      <c r="G23" s="41" t="inlineStr">
+      <c r="B23" s="60" t="n"/>
+      <c r="C23" s="61" t="n"/>
+      <c r="D23" s="62" t="n"/>
+      <c r="E23" s="63" t="n"/>
+      <c r="F23" s="64" t="n"/>
+      <c r="G23" s="65" t="inlineStr">
         <is>
           <t>MTR</t>
         </is>
       </c>
-      <c r="H23" s="41" t="inlineStr">
+      <c r="H23" s="66" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="O23" s="41" t="inlineStr">
+      <c r="I23" s="67" t="n"/>
+      <c r="J23" s="68" t="n"/>
+      <c r="K23" s="69" t="n"/>
+      <c r="L23" s="70" t="n"/>
+      <c r="M23" s="71" t="n"/>
+      <c r="N23" s="72" t="n"/>
+      <c r="O23" s="73" t="inlineStr">
         <is>
           <t>MTR</t>
         </is>
       </c>
-      <c r="P23" s="41" t="inlineStr">
+      <c r="P23" s="74" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="Q23" s="41" t="inlineStr">
+      <c r="Q23" s="75" t="inlineStr">
         <is>
           <t>MTR</t>
         </is>
       </c>
-      <c r="R23" s="41" t="inlineStr">
+      <c r="R23" s="76" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
+      <c r="S23" s="77" t="n"/>
+      <c r="T23" s="78" t="n"/>
     </row>
     <row r="24">
-      <c r="G24" s="41" t="inlineStr">
+      <c r="B24" s="60" t="n"/>
+      <c r="C24" s="61" t="n"/>
+      <c r="D24" s="62" t="n"/>
+      <c r="E24" s="63" t="n"/>
+      <c r="F24" s="64" t="n"/>
+      <c r="G24" s="65" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="H24" s="41" t="inlineStr">
+      <c r="H24" s="66" t="inlineStr">
         <is>
           <t>10.4</t>
         </is>
       </c>
-      <c r="O24" s="41" t="inlineStr">
+      <c r="I24" s="67" t="n"/>
+      <c r="J24" s="68" t="n"/>
+      <c r="K24" s="69" t="n"/>
+      <c r="L24" s="70" t="n"/>
+      <c r="M24" s="71" t="n"/>
+      <c r="N24" s="72" t="n"/>
+      <c r="O24" s="73" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="P24" s="41" t="inlineStr">
+      <c r="P24" s="74" t="inlineStr">
         <is>
           <t>10.4</t>
         </is>
       </c>
-      <c r="Q24" s="41" t="inlineStr">
+      <c r="Q24" s="75" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="R24" s="41" t="inlineStr">
+      <c r="R24" s="76" t="inlineStr">
         <is>
           <t>10.4</t>
         </is>
       </c>
+      <c r="S24" s="77" t="n"/>
+      <c r="T24" s="78" t="n"/>
     </row>
     <row r="25">
-      <c r="E25" s="41" t="inlineStr">
+      <c r="B25" s="60" t="n"/>
+      <c r="C25" s="61" t="n"/>
+      <c r="D25" s="62" t="n"/>
+      <c r="E25" s="79" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F25" s="41" t="inlineStr">
+      <c r="F25" s="80" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
-      <c r="I25" s="41" t="inlineStr">
+      <c r="G25" s="81" t="n"/>
+      <c r="H25" s="82" t="n"/>
+      <c r="I25" s="83" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
-      <c r="J25" s="41" t="inlineStr">
+      <c r="J25" s="84" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="K25" s="69" t="n"/>
+      <c r="L25" s="70" t="n"/>
+      <c r="M25" s="71" t="n"/>
+      <c r="N25" s="72" t="n"/>
+      <c r="O25" s="85" t="n"/>
+      <c r="P25" s="86" t="n"/>
+      <c r="Q25" s="87" t="n"/>
+      <c r="R25" s="88" t="n"/>
+      <c r="S25" s="77" t="n"/>
+      <c r="T25" s="78" t="n"/>
     </row>
     <row r="26">
-      <c r="I26" s="41" t="inlineStr">
+      <c r="B26" s="60" t="n"/>
+      <c r="C26" s="61" t="n"/>
+      <c r="D26" s="62" t="n"/>
+      <c r="E26" s="63" t="n"/>
+      <c r="F26" s="64" t="n"/>
+      <c r="G26" s="81" t="n"/>
+      <c r="H26" s="82" t="n"/>
+      <c r="I26" s="83" t="inlineStr">
         <is>
           <t>Piggy</t>
         </is>
       </c>
-      <c r="J26" s="41" t="inlineStr">
+      <c r="J26" s="84" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
-      <c r="O26" s="41" t="inlineStr">
+      <c r="K26" s="69" t="n"/>
+      <c r="L26" s="70" t="n"/>
+      <c r="M26" s="71" t="n"/>
+      <c r="N26" s="72" t="n"/>
+      <c r="O26" s="73" t="inlineStr">
         <is>
           <t>Piggy</t>
         </is>
       </c>
-      <c r="P26" s="41" t="inlineStr">
+      <c r="P26" s="74" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
-      <c r="Q26" s="41" t="inlineStr">
+      <c r="Q26" s="75" t="inlineStr">
         <is>
           <t>Piggy</t>
         </is>
       </c>
-      <c r="R26" s="41" t="inlineStr">
+      <c r="R26" s="76" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
+      <c r="S26" s="77" t="n"/>
+      <c r="T26" s="78" t="n"/>
     </row>
     <row r="27">
-      <c r="E27" s="41" t="inlineStr">
+      <c r="B27" s="60" t="n"/>
+      <c r="C27" s="61" t="n"/>
+      <c r="D27" s="62" t="n"/>
+      <c r="E27" s="79" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F27" s="41" t="inlineStr">
+      <c r="F27" s="80" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="I27" s="41" t="inlineStr">
+      <c r="G27" s="81" t="n"/>
+      <c r="H27" s="82" t="n"/>
+      <c r="I27" s="83" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="J27" s="41" t="inlineStr">
+      <c r="J27" s="84" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="K27" s="69" t="n"/>
+      <c r="L27" s="70" t="n"/>
+      <c r="M27" s="71" t="n"/>
+      <c r="N27" s="72" t="n"/>
+      <c r="O27" s="85" t="n"/>
+      <c r="P27" s="86" t="n"/>
+      <c r="Q27" s="87" t="n"/>
+      <c r="R27" s="88" t="n"/>
+      <c r="S27" s="77" t="n"/>
+      <c r="T27" s="78" t="n"/>
     </row>
     <row r="28">
-      <c r="I28" s="41" t="inlineStr">
+      <c r="B28" s="60" t="n"/>
+      <c r="C28" s="61" t="n"/>
+      <c r="D28" s="62" t="n"/>
+      <c r="E28" s="63" t="n"/>
+      <c r="F28" s="64" t="n"/>
+      <c r="G28" s="81" t="n"/>
+      <c r="H28" s="82" t="n"/>
+      <c r="I28" s="83" t="inlineStr">
         <is>
           <t>Piggy play</t>
         </is>
       </c>
-      <c r="J28" s="41" t="inlineStr">
+      <c r="J28" s="84" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="O28" s="41" t="inlineStr">
+      <c r="K28" s="69" t="n"/>
+      <c r="L28" s="70" t="n"/>
+      <c r="M28" s="71" t="n"/>
+      <c r="N28" s="72" t="n"/>
+      <c r="O28" s="73" t="inlineStr">
         <is>
           <t>Piggy play</t>
         </is>
       </c>
-      <c r="P28" s="41" t="inlineStr">
+      <c r="P28" s="74" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="Q28" s="41" t="inlineStr">
+      <c r="Q28" s="75" t="inlineStr">
         <is>
           <t>Piggy play</t>
         </is>
       </c>
-      <c r="R28" s="41" t="inlineStr">
+      <c r="R28" s="76" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
+      <c r="S28" s="77" t="n"/>
+      <c r="T28" s="78" t="n"/>
     </row>
     <row r="29">
-      <c r="E29" s="41" t="inlineStr">
+      <c r="B29" s="60" t="n"/>
+      <c r="C29" s="61" t="n"/>
+      <c r="D29" s="62" t="n"/>
+      <c r="E29" s="79" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F29" s="41" t="inlineStr">
+      <c r="F29" s="80" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="I29" s="41" t="inlineStr">
+      <c r="G29" s="81" t="n"/>
+      <c r="H29" s="82" t="n"/>
+      <c r="I29" s="83" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="J29" s="41" t="inlineStr">
+      <c r="J29" s="84" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="K29" s="69" t="n"/>
+      <c r="L29" s="70" t="n"/>
+      <c r="M29" s="71" t="n"/>
+      <c r="N29" s="72" t="n"/>
+      <c r="O29" s="85" t="n"/>
+      <c r="P29" s="86" t="n"/>
+      <c r="Q29" s="87" t="n"/>
+      <c r="R29" s="88" t="n"/>
+      <c r="S29" s="77" t="n"/>
+      <c r="T29" s="78" t="n"/>
     </row>
     <row r="30">
-      <c r="I30" s="41" t="inlineStr">
+      <c r="B30" s="60" t="n"/>
+      <c r="C30" s="61" t="n"/>
+      <c r="D30" s="62" t="n"/>
+      <c r="E30" s="63" t="n"/>
+      <c r="F30" s="64" t="n"/>
+      <c r="G30" s="81" t="n"/>
+      <c r="H30" s="82" t="n"/>
+      <c r="I30" s="83" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="J30" s="41" t="inlineStr">
+      <c r="J30" s="84" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="O30" s="41" t="inlineStr">
+      <c r="K30" s="69" t="n"/>
+      <c r="L30" s="70" t="n"/>
+      <c r="M30" s="71" t="n"/>
+      <c r="N30" s="72" t="n"/>
+      <c r="O30" s="73" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="P30" s="41" t="inlineStr">
+      <c r="P30" s="74" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="Q30" s="41" t="inlineStr">
+      <c r="Q30" s="75" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="R30" s="41" t="inlineStr">
+      <c r="R30" s="76" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
+      <c r="S30" s="77" t="n"/>
+      <c r="T30" s="78" t="n"/>
     </row>
     <row r="31">
-      <c r="E31" s="41" t="inlineStr">
+      <c r="B31" s="60" t="n"/>
+      <c r="C31" s="61" t="n"/>
+      <c r="D31" s="62" t="n"/>
+      <c r="E31" s="79" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F31" s="41" t="inlineStr">
+      <c r="F31" s="80" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
-      <c r="I31" s="41" t="inlineStr">
+      <c r="G31" s="81" t="n"/>
+      <c r="H31" s="82" t="n"/>
+      <c r="I31" s="83" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
-      <c r="J31" s="41" t="inlineStr">
+      <c r="J31" s="84" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="K31" s="69" t="n"/>
+      <c r="L31" s="70" t="n"/>
+      <c r="M31" s="71" t="n"/>
+      <c r="N31" s="72" t="n"/>
+      <c r="O31" s="85" t="n"/>
+      <c r="P31" s="86" t="n"/>
+      <c r="Q31" s="87" t="n"/>
+      <c r="R31" s="88" t="n"/>
+      <c r="S31" s="77" t="n"/>
+      <c r="T31" s="78" t="n"/>
     </row>
     <row r="32">
-      <c r="I32" s="41" t="inlineStr">
+      <c r="B32" s="60" t="n"/>
+      <c r="C32" s="61" t="n"/>
+      <c r="D32" s="62" t="n"/>
+      <c r="E32" s="63" t="n"/>
+      <c r="F32" s="64" t="n"/>
+      <c r="G32" s="81" t="n"/>
+      <c r="H32" s="82" t="n"/>
+      <c r="I32" s="83" t="inlineStr">
         <is>
           <t>Dinner</t>
         </is>
       </c>
-      <c r="J32" s="41" t="inlineStr">
+      <c r="J32" s="84" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
-      <c r="O32" s="41" t="inlineStr">
+      <c r="K32" s="69" t="n"/>
+      <c r="L32" s="70" t="n"/>
+      <c r="M32" s="71" t="n"/>
+      <c r="N32" s="72" t="n"/>
+      <c r="O32" s="73" t="inlineStr">
         <is>
           <t>Dinner</t>
         </is>
       </c>
-      <c r="P32" s="41" t="inlineStr">
+      <c r="P32" s="74" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
-      <c r="Q32" s="41" t="inlineStr">
+      <c r="Q32" s="75" t="inlineStr">
         <is>
           <t>Dinner</t>
         </is>
       </c>
-      <c r="R32" s="41" t="inlineStr">
+      <c r="R32" s="76" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
+      <c r="S32" s="77" t="n"/>
+      <c r="T32" s="78" t="n"/>
     </row>
     <row r="33">
-      <c r="C33" s="41" t="inlineStr">
+      <c r="B33" s="60" t="n"/>
+      <c r="C33" s="154" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="D33" s="41" t="inlineStr">
+      <c r="D33" s="155" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
-      <c r="O33" s="41" t="inlineStr">
+      <c r="E33" s="63" t="n"/>
+      <c r="F33" s="64" t="n"/>
+      <c r="G33" s="81" t="n"/>
+      <c r="H33" s="82" t="n"/>
+      <c r="I33" s="67" t="n"/>
+      <c r="J33" s="68" t="n"/>
+      <c r="K33" s="69" t="n"/>
+      <c r="L33" s="70" t="n"/>
+      <c r="M33" s="71" t="n"/>
+      <c r="N33" s="72" t="n"/>
+      <c r="O33" s="73" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="P33" s="41" t="inlineStr">
+      <c r="P33" s="74" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
-      <c r="Q33" s="41" t="inlineStr">
+      <c r="Q33" s="75" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="R33" s="41" t="inlineStr">
+      <c r="R33" s="76" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
+      <c r="S33" s="77" t="n"/>
+      <c r="T33" s="78" t="n"/>
     </row>
     <row r="34">
-      <c r="C34" s="41" t="inlineStr">
+      <c r="B34" s="60" t="n"/>
+      <c r="C34" s="154" t="inlineStr">
         <is>
           <t>Coin hold</t>
         </is>
       </c>
-      <c r="D34" s="41" t="inlineStr">
+      <c r="D34" s="155" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="O34" s="41" t="inlineStr">
+      <c r="E34" s="63" t="n"/>
+      <c r="F34" s="64" t="n"/>
+      <c r="G34" s="81" t="n"/>
+      <c r="H34" s="82" t="n"/>
+      <c r="I34" s="67" t="n"/>
+      <c r="J34" s="68" t="n"/>
+      <c r="K34" s="69" t="n"/>
+      <c r="L34" s="70" t="n"/>
+      <c r="M34" s="71" t="n"/>
+      <c r="N34" s="72" t="n"/>
+      <c r="O34" s="73" t="inlineStr">
         <is>
           <t>Coin hold</t>
         </is>
       </c>
-      <c r="P34" s="41" t="inlineStr">
+      <c r="P34" s="74" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="Q34" s="41" t="inlineStr">
+      <c r="Q34" s="75" t="inlineStr">
         <is>
           <t>Coin hold</t>
         </is>
       </c>
-      <c r="R34" s="41" t="inlineStr">
+      <c r="R34" s="76" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
+      <c r="S34" s="77" t="n"/>
+      <c r="T34" s="78" t="n"/>
     </row>
     <row r="35">
-      <c r="E35" s="41" t="inlineStr">
+      <c r="B35" s="91" t="n"/>
+      <c r="C35" s="92" t="n"/>
+      <c r="D35" s="93" t="n"/>
+      <c r="E35" s="156" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="F35" s="41" t="inlineStr">
+      <c r="F35" s="157" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="G35" s="41" t="inlineStr">
+      <c r="G35" s="158" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="H35" s="41" t="inlineStr">
+      <c r="H35" s="159" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
+      <c r="I35" s="160" t="n"/>
+      <c r="J35" s="161" t="n"/>
+      <c r="K35" s="100" t="n"/>
+      <c r="L35" s="101" t="n"/>
+      <c r="M35" s="102" t="n"/>
+      <c r="N35" s="103" t="n"/>
+      <c r="O35" s="162" t="n"/>
+      <c r="P35" s="163" t="n"/>
+      <c r="Q35" s="164" t="n"/>
+      <c r="R35" s="165" t="n"/>
+      <c r="S35" s="108" t="n"/>
+      <c r="T35" s="109" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="41" t="inlineStr">
+      <c r="B36" s="110" t="inlineStr">
         <is>
           <t>sum</t>
         </is>
       </c>
-      <c r="C36" s="41" t="n">
+      <c r="C36" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="E36" s="41" t="n">
+      <c r="D36" s="112" t="n"/>
+      <c r="E36" s="113" t="n">
         <v>15595.12</v>
       </c>
-      <c r="G36" s="41" t="n">
+      <c r="F36" s="114" t="n"/>
+      <c r="G36" s="115" t="n">
         <v>541</v>
       </c>
-      <c r="I36" s="41" t="n">
+      <c r="H36" s="116" t="n"/>
+      <c r="I36" s="117" t="n">
         <v>0</v>
       </c>
-      <c r="K36" s="41" t="n">
+      <c r="J36" s="118" t="n"/>
+      <c r="K36" s="119" t="n">
         <v>0</v>
       </c>
-      <c r="M36" s="41" t="n">
+      <c r="L36" s="120" t="n"/>
+      <c r="M36" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="O36" s="41" t="n">
+      <c r="N36" s="122" t="n"/>
+      <c r="O36" s="123" t="n">
         <v>0</v>
       </c>
-      <c r="P36" s="41" t="n">
+      <c r="P36" s="124" t="n">
         <v>2953.1</v>
       </c>
-      <c r="Q36" s="41" t="n">
+      <c r="Q36" s="125" t="n">
         <v>7000</v>
       </c>
-      <c r="R36" s="41" t="n">
+      <c r="R36" s="126" t="n">
         <v>5946.1</v>
       </c>
-      <c r="S36" s="41" t="n">
+      <c r="S36" s="127" t="n">
         <v>16136.12</v>
       </c>
-      <c r="T36" s="41" t="inlineStr">
+      <c r="T36" s="128" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="41" t="inlineStr">
+      <c r="B37" s="129" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="O37" s="41" t="n">
+      <c r="C37" s="130" t="n"/>
+      <c r="D37" s="131" t="n"/>
+      <c r="E37" s="132" t="n"/>
+      <c r="F37" s="133" t="n"/>
+      <c r="G37" s="134" t="n"/>
+      <c r="H37" s="135" t="n"/>
+      <c r="I37" s="136" t="n"/>
+      <c r="J37" s="137" t="n"/>
+      <c r="K37" s="138" t="n"/>
+      <c r="L37" s="139" t="n"/>
+      <c r="M37" s="140" t="n"/>
+      <c r="N37" s="141" t="n"/>
+      <c r="O37" s="142" t="n">
         <v>0</v>
       </c>
-      <c r="P37" s="41" t="n">
+      <c r="P37" s="143" t="n">
         <v>3296.8</v>
       </c>
-      <c r="Q37" s="41" t="n">
+      <c r="Q37" s="144" t="n">
         <v>7000</v>
       </c>
-      <c r="R37" s="41" t="n">
+      <c r="R37" s="145" t="n">
         <v>6289.8</v>
       </c>
+      <c r="S37" s="146" t="n"/>
+      <c r="T37" s="147" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="41" t="inlineStr">
+      <c r="B38" s="1" t="inlineStr">
         <is>
           <t>current have</t>
         </is>
       </c>
-      <c r="C38" s="41" t="n">
+      <c r="C38" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="41" t="inlineStr">
+      <c r="D38" s="14" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="E38" s="41" t="n">
+      <c r="E38" s="15" t="n">
         <v>15595.12</v>
       </c>
-      <c r="F38" s="41" t="inlineStr">
+      <c r="F38" s="16" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="G38" s="41" t="n">
+      <c r="G38" s="17" t="n">
         <v>541</v>
       </c>
-      <c r="H38" s="41" t="inlineStr">
+      <c r="H38" s="18" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I38" s="41" t="n">
+      <c r="I38" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="J38" s="41" t="inlineStr">
+      <c r="J38" s="20" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="K38" s="41" t="n">
+      <c r="K38" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="L38" s="41" t="inlineStr">
+      <c r="L38" s="22" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="M38" s="41" t="n">
+      <c r="M38" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="N38" s="41" t="inlineStr">
+      <c r="N38" s="24" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="S38" s="41" t="n">
+      <c r="O38" s="37" t="n"/>
+      <c r="P38" s="38" t="n"/>
+      <c r="Q38" s="39" t="n"/>
+      <c r="R38" s="40" t="n"/>
+      <c r="S38" s="29" t="n">
         <v>16136.12</v>
       </c>
+      <c r="T38" s="30" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
add coin-hold col in money excel
</commit_message>
<xml_diff>
--- a/output/2026/money.xlsx
+++ b/output/2026/money.xlsx
@@ -31,7 +31,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EBF1DE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
     <fill>
@@ -268,7 +273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="183">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -296,8 +301,11 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -313,69 +321,76 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -383,18 +398,20 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -409,11 +426,13 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -427,30 +446,35 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -829,7 +853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T38"/>
+  <dimension ref="A2:V38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.5" customWidth="1" min="2" max="2"/>
@@ -851,6 +875,8 @@
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -867,48 +893,54 @@
       <c r="D2" s="3" t="n"/>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>Coin-hold</t>
         </is>
       </c>
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Octopus</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>AliPay</t>
+          <t>Octopus</t>
         </is>
       </c>
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Tap and Go</t>
+          <t>AliPay</t>
         </is>
       </c>
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="8" t="inlineStr">
         <is>
-          <t>Payme</t>
+          <t>Tap and Go</t>
         </is>
       </c>
       <c r="N2" s="3" t="n"/>
       <c r="O2" s="9" t="inlineStr">
         <is>
-          <t>Countable Total</t>
+          <t>Payme</t>
         </is>
       </c>
       <c r="P2" s="3" t="n"/>
       <c r="Q2" s="10" t="inlineStr">
         <is>
+          <t>Countable Total</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="n"/>
+      <c r="S2" s="11" t="inlineStr">
+        <is>
           <t>Real Total</t>
         </is>
       </c>
-      <c r="R2" s="11" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="12" t="inlineStr">
+      <c r="T2" s="12" t="n"/>
+      <c r="U2" s="3" t="n"/>
+      <c r="V2" s="13" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -920,92 +952,102 @@
           <t>DD/MM/YY</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="E3" s="15" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="G3" s="17" t="inlineStr">
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="H3" s="18" t="inlineStr">
+      <c r="H3" s="19" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="I3" s="19" t="inlineStr">
+      <c r="I3" s="20" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="J3" s="20" t="inlineStr">
+      <c r="J3" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="K3" s="21" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="L3" s="22" t="inlineStr">
+      <c r="L3" s="23" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="M3" s="23" t="inlineStr">
+      <c r="M3" s="24" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="N3" s="24" t="inlineStr">
+      <c r="N3" s="25" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="O3" s="25" t="inlineStr">
+      <c r="O3" s="26" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="P3" s="26" t="inlineStr">
+      <c r="P3" s="27" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="Q3" s="27" t="inlineStr">
+      <c r="Q3" s="28" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="R3" s="28" t="inlineStr">
+      <c r="R3" s="29" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="S3" s="29" t="inlineStr">
+      <c r="S3" s="30" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="T3" s="31" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="U3" s="32" t="inlineStr">
         <is>
           <t>Have</t>
         </is>
       </c>
-      <c r="T3" s="30" t="n"/>
+      <c r="V3" s="33" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="1" t="inlineStr">
@@ -1013,1429 +1055,1497 @@
           <t>Last</t>
         </is>
       </c>
-      <c r="C4" s="13" t="n">
+      <c r="C4" s="14" t="n">
         <v>70</v>
       </c>
-      <c r="D4" s="31" t="n"/>
-      <c r="E4" s="15" t="n">
+      <c r="D4" s="34" t="n"/>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="n"/>
+      <c r="G4" s="18" t="n">
         <v>15266.02</v>
       </c>
-      <c r="F4" s="32" t="n"/>
-      <c r="G4" s="17" t="n">
+      <c r="H4" s="36" t="n"/>
+      <c r="I4" s="20" t="n">
         <v>89.90000000000001</v>
       </c>
-      <c r="H4" s="33" t="n"/>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="J4" s="37" t="n"/>
+      <c r="K4" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J4" s="34" t="n"/>
-      <c r="K4" s="21" t="inlineStr">
+      <c r="L4" s="38" t="n"/>
+      <c r="M4" s="24" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L4" s="35" t="n"/>
-      <c r="M4" s="23" t="inlineStr">
+      <c r="N4" s="39" t="n"/>
+      <c r="O4" s="26" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N4" s="36" t="n"/>
-      <c r="O4" s="37" t="n"/>
-      <c r="P4" s="38" t="n"/>
-      <c r="Q4" s="39" t="n"/>
-      <c r="R4" s="40" t="n"/>
-      <c r="S4" s="29" t="n">
+      <c r="P4" s="40" t="n"/>
+      <c r="Q4" s="41" t="n"/>
+      <c r="R4" s="42" t="n"/>
+      <c r="S4" s="43" t="n"/>
+      <c r="T4" s="44" t="n"/>
+      <c r="U4" s="32" t="n">
         <v>15425.92</v>
       </c>
-      <c r="T4" s="30" t="n"/>
+      <c r="V4" s="33" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="41" t="inlineStr">
+      <c r="B5" s="45" t="inlineStr">
         <is>
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="C5" s="42" t="n"/>
-      <c r="D5" s="43" t="n"/>
-      <c r="E5" s="44" t="n"/>
-      <c r="F5" s="45" t="n"/>
-      <c r="G5" s="46" t="inlineStr">
+      <c r="C5" s="46" t="n"/>
+      <c r="D5" s="47" t="n"/>
+      <c r="E5" s="48" t="n"/>
+      <c r="F5" s="49" t="n"/>
+      <c r="G5" s="50" t="n"/>
+      <c r="H5" s="51" t="n"/>
+      <c r="I5" s="52" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="H5" s="47" t="inlineStr">
+      <c r="J5" s="53" t="inlineStr">
         <is>
           <t>14.6</t>
         </is>
       </c>
-      <c r="I5" s="48" t="n"/>
-      <c r="J5" s="49" t="n"/>
-      <c r="K5" s="50" t="n"/>
-      <c r="L5" s="51" t="n"/>
-      <c r="M5" s="52" t="n"/>
-      <c r="N5" s="53" t="n"/>
-      <c r="O5" s="54" t="inlineStr">
+      <c r="K5" s="54" t="n"/>
+      <c r="L5" s="55" t="n"/>
+      <c r="M5" s="56" t="n"/>
+      <c r="N5" s="57" t="n"/>
+      <c r="O5" s="58" t="n"/>
+      <c r="P5" s="59" t="n"/>
+      <c r="Q5" s="60" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="P5" s="55" t="inlineStr">
+      <c r="R5" s="61" t="inlineStr">
         <is>
           <t>14.6</t>
         </is>
       </c>
-      <c r="Q5" s="56" t="inlineStr">
+      <c r="S5" s="62" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="R5" s="57" t="inlineStr">
+      <c r="T5" s="63" t="inlineStr">
         <is>
           <t>14.6</t>
         </is>
       </c>
-      <c r="S5" s="58" t="n"/>
-      <c r="T5" s="59" t="n"/>
+      <c r="U5" s="64" t="n"/>
+      <c r="V5" s="65" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="60" t="n"/>
-      <c r="C6" s="61" t="n"/>
-      <c r="D6" s="62" t="n"/>
-      <c r="E6" s="63" t="n"/>
-      <c r="F6" s="64" t="n"/>
-      <c r="G6" s="65" t="inlineStr">
+      <c r="B6" s="66" t="n"/>
+      <c r="C6" s="67" t="n"/>
+      <c r="D6" s="68" t="n"/>
+      <c r="E6" s="69" t="n"/>
+      <c r="F6" s="70" t="n"/>
+      <c r="G6" s="71" t="n"/>
+      <c r="H6" s="72" t="n"/>
+      <c r="I6" s="73" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="H6" s="66" t="inlineStr">
+      <c r="J6" s="74" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="I6" s="67" t="n"/>
-      <c r="J6" s="68" t="n"/>
-      <c r="K6" s="69" t="n"/>
-      <c r="L6" s="70" t="n"/>
-      <c r="M6" s="71" t="n"/>
-      <c r="N6" s="72" t="n"/>
-      <c r="O6" s="73" t="inlineStr">
+      <c r="K6" s="75" t="n"/>
+      <c r="L6" s="76" t="n"/>
+      <c r="M6" s="77" t="n"/>
+      <c r="N6" s="78" t="n"/>
+      <c r="O6" s="79" t="n"/>
+      <c r="P6" s="80" t="n"/>
+      <c r="Q6" s="81" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="P6" s="74" t="inlineStr">
+      <c r="R6" s="82" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="Q6" s="75" t="inlineStr">
+      <c r="S6" s="83" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="R6" s="76" t="inlineStr">
+      <c r="T6" s="84" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="S6" s="77" t="n"/>
-      <c r="T6" s="78" t="n"/>
+      <c r="U6" s="85" t="n"/>
+      <c r="V6" s="86" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="60" t="n"/>
-      <c r="C7" s="61" t="n"/>
-      <c r="D7" s="62" t="n"/>
-      <c r="E7" s="79" t="inlineStr">
+      <c r="B7" s="66" t="n"/>
+      <c r="C7" s="67" t="n"/>
+      <c r="D7" s="68" t="n"/>
+      <c r="E7" s="69" t="n"/>
+      <c r="F7" s="70" t="n"/>
+      <c r="G7" s="87" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F7" s="80" t="inlineStr">
+      <c r="H7" s="88" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="G7" s="81" t="n"/>
-      <c r="H7" s="82" t="n"/>
-      <c r="I7" s="83" t="inlineStr">
+      <c r="I7" s="89" t="n"/>
+      <c r="J7" s="90" t="n"/>
+      <c r="K7" s="91" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="J7" s="84" t="inlineStr">
+      <c r="L7" s="92" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K7" s="69" t="n"/>
-      <c r="L7" s="70" t="n"/>
-      <c r="M7" s="71" t="n"/>
-      <c r="N7" s="72" t="n"/>
-      <c r="O7" s="85" t="n"/>
-      <c r="P7" s="86" t="n"/>
-      <c r="Q7" s="87" t="n"/>
-      <c r="R7" s="88" t="n"/>
-      <c r="S7" s="77" t="n"/>
-      <c r="T7" s="78" t="n"/>
+      <c r="M7" s="77" t="n"/>
+      <c r="N7" s="78" t="n"/>
+      <c r="O7" s="79" t="n"/>
+      <c r="P7" s="80" t="n"/>
+      <c r="Q7" s="93" t="n"/>
+      <c r="R7" s="94" t="n"/>
+      <c r="S7" s="95" t="n"/>
+      <c r="T7" s="96" t="n"/>
+      <c r="U7" s="85" t="n"/>
+      <c r="V7" s="86" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="60" t="n"/>
-      <c r="C8" s="61" t="n"/>
-      <c r="D8" s="62" t="n"/>
-      <c r="E8" s="63" t="n"/>
-      <c r="F8" s="64" t="n"/>
-      <c r="G8" s="81" t="n"/>
-      <c r="H8" s="82" t="n"/>
-      <c r="I8" s="83" t="inlineStr">
+      <c r="B8" s="66" t="n"/>
+      <c r="C8" s="67" t="n"/>
+      <c r="D8" s="68" t="n"/>
+      <c r="E8" s="69" t="n"/>
+      <c r="F8" s="70" t="n"/>
+      <c r="G8" s="71" t="n"/>
+      <c r="H8" s="72" t="n"/>
+      <c r="I8" s="89" t="n"/>
+      <c r="J8" s="90" t="n"/>
+      <c r="K8" s="91" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="J8" s="84" t="inlineStr">
+      <c r="L8" s="92" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="K8" s="69" t="n"/>
-      <c r="L8" s="70" t="n"/>
-      <c r="M8" s="71" t="n"/>
-      <c r="N8" s="72" t="n"/>
-      <c r="O8" s="73" t="inlineStr">
+      <c r="M8" s="77" t="n"/>
+      <c r="N8" s="78" t="n"/>
+      <c r="O8" s="79" t="n"/>
+      <c r="P8" s="80" t="n"/>
+      <c r="Q8" s="81" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="P8" s="74" t="inlineStr">
+      <c r="R8" s="82" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="Q8" s="75" t="inlineStr">
+      <c r="S8" s="83" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="R8" s="76" t="inlineStr">
+      <c r="T8" s="84" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="S8" s="77" t="n"/>
-      <c r="T8" s="78" t="n"/>
+      <c r="U8" s="85" t="n"/>
+      <c r="V8" s="86" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="60" t="n"/>
-      <c r="C9" s="61" t="n"/>
-      <c r="D9" s="62" t="n"/>
-      <c r="E9" s="79" t="inlineStr">
+      <c r="B9" s="66" t="n"/>
+      <c r="C9" s="67" t="n"/>
+      <c r="D9" s="68" t="n"/>
+      <c r="E9" s="69" t="n"/>
+      <c r="F9" s="70" t="n"/>
+      <c r="G9" s="87" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F9" s="80" t="inlineStr">
+      <c r="H9" s="88" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
-      <c r="G9" s="81" t="n"/>
-      <c r="H9" s="82" t="n"/>
-      <c r="I9" s="83" t="inlineStr">
+      <c r="I9" s="89" t="n"/>
+      <c r="J9" s="90" t="n"/>
+      <c r="K9" s="91" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
-      <c r="J9" s="84" t="inlineStr">
+      <c r="L9" s="92" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K9" s="69" t="n"/>
-      <c r="L9" s="70" t="n"/>
-      <c r="M9" s="71" t="n"/>
-      <c r="N9" s="72" t="n"/>
-      <c r="O9" s="85" t="n"/>
-      <c r="P9" s="86" t="n"/>
-      <c r="Q9" s="87" t="n"/>
-      <c r="R9" s="88" t="n"/>
-      <c r="S9" s="77" t="n"/>
-      <c r="T9" s="78" t="n"/>
+      <c r="M9" s="77" t="n"/>
+      <c r="N9" s="78" t="n"/>
+      <c r="O9" s="79" t="n"/>
+      <c r="P9" s="80" t="n"/>
+      <c r="Q9" s="93" t="n"/>
+      <c r="R9" s="94" t="n"/>
+      <c r="S9" s="95" t="n"/>
+      <c r="T9" s="96" t="n"/>
+      <c r="U9" s="85" t="n"/>
+      <c r="V9" s="86" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="60" t="n"/>
-      <c r="C10" s="61" t="n"/>
-      <c r="D10" s="62" t="n"/>
-      <c r="E10" s="63" t="n"/>
-      <c r="F10" s="64" t="n"/>
-      <c r="G10" s="81" t="n"/>
-      <c r="H10" s="82" t="n"/>
-      <c r="I10" s="83" t="inlineStr">
+      <c r="B10" s="66" t="n"/>
+      <c r="C10" s="67" t="n"/>
+      <c r="D10" s="68" t="n"/>
+      <c r="E10" s="69" t="n"/>
+      <c r="F10" s="70" t="n"/>
+      <c r="G10" s="71" t="n"/>
+      <c r="H10" s="72" t="n"/>
+      <c r="I10" s="89" t="n"/>
+      <c r="J10" s="90" t="n"/>
+      <c r="K10" s="91" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="J10" s="84" t="inlineStr">
+      <c r="L10" s="92" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
-      <c r="K10" s="69" t="n"/>
-      <c r="L10" s="70" t="n"/>
-      <c r="M10" s="71" t="n"/>
-      <c r="N10" s="72" t="n"/>
-      <c r="O10" s="73" t="inlineStr">
+      <c r="M10" s="77" t="n"/>
+      <c r="N10" s="78" t="n"/>
+      <c r="O10" s="79" t="n"/>
+      <c r="P10" s="80" t="n"/>
+      <c r="Q10" s="81" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="P10" s="74" t="inlineStr">
+      <c r="R10" s="82" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
-      <c r="Q10" s="75" t="inlineStr">
+      <c r="S10" s="83" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="R10" s="76" t="inlineStr">
+      <c r="T10" s="84" t="inlineStr">
         <is>
           <t>184</t>
         </is>
       </c>
-      <c r="S10" s="77" t="n"/>
-      <c r="T10" s="78" t="n"/>
+      <c r="U10" s="85" t="n"/>
+      <c r="V10" s="86" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="60" t="n"/>
-      <c r="C11" s="61" t="n"/>
-      <c r="D11" s="62" t="n"/>
-      <c r="E11" s="79" t="inlineStr">
+      <c r="B11" s="66" t="n"/>
+      <c r="C11" s="67" t="n"/>
+      <c r="D11" s="68" t="n"/>
+      <c r="E11" s="69" t="n"/>
+      <c r="F11" s="70" t="n"/>
+      <c r="G11" s="87" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F11" s="80" t="inlineStr">
+      <c r="H11" s="88" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="G11" s="81" t="n"/>
-      <c r="H11" s="82" t="n"/>
-      <c r="I11" s="67" t="n"/>
-      <c r="J11" s="68" t="n"/>
-      <c r="K11" s="69" t="n"/>
-      <c r="L11" s="70" t="n"/>
-      <c r="M11" s="89" t="inlineStr">
+      <c r="I11" s="89" t="n"/>
+      <c r="J11" s="90" t="n"/>
+      <c r="K11" s="75" t="n"/>
+      <c r="L11" s="76" t="n"/>
+      <c r="M11" s="77" t="n"/>
+      <c r="N11" s="78" t="n"/>
+      <c r="O11" s="97" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="N11" s="90" t="inlineStr">
+      <c r="P11" s="98" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="O11" s="85" t="n"/>
-      <c r="P11" s="86" t="n"/>
-      <c r="Q11" s="87" t="n"/>
-      <c r="R11" s="88" t="n"/>
-      <c r="S11" s="77" t="n"/>
-      <c r="T11" s="78" t="n"/>
+      <c r="Q11" s="93" t="n"/>
+      <c r="R11" s="94" t="n"/>
+      <c r="S11" s="95" t="n"/>
+      <c r="T11" s="96" t="n"/>
+      <c r="U11" s="85" t="n"/>
+      <c r="V11" s="86" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="60" t="n"/>
-      <c r="C12" s="61" t="n"/>
-      <c r="D12" s="62" t="n"/>
-      <c r="E12" s="63" t="n"/>
-      <c r="F12" s="64" t="n"/>
-      <c r="G12" s="81" t="n"/>
-      <c r="H12" s="82" t="n"/>
-      <c r="I12" s="67" t="n"/>
-      <c r="J12" s="68" t="n"/>
-      <c r="K12" s="69" t="n"/>
-      <c r="L12" s="70" t="n"/>
-      <c r="M12" s="89" t="inlineStr">
+      <c r="B12" s="66" t="n"/>
+      <c r="C12" s="67" t="n"/>
+      <c r="D12" s="68" t="n"/>
+      <c r="E12" s="69" t="n"/>
+      <c r="F12" s="70" t="n"/>
+      <c r="G12" s="71" t="n"/>
+      <c r="H12" s="72" t="n"/>
+      <c r="I12" s="89" t="n"/>
+      <c r="J12" s="90" t="n"/>
+      <c r="K12" s="75" t="n"/>
+      <c r="L12" s="76" t="n"/>
+      <c r="M12" s="77" t="n"/>
+      <c r="N12" s="78" t="n"/>
+      <c r="O12" s="97" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="N12" s="90" t="inlineStr">
+      <c r="P12" s="98" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="O12" s="73" t="inlineStr">
+      <c r="Q12" s="81" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="P12" s="74" t="inlineStr">
+      <c r="R12" s="82" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="Q12" s="75" t="inlineStr">
+      <c r="S12" s="83" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="R12" s="76" t="inlineStr">
+      <c r="T12" s="84" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="S12" s="77" t="n"/>
-      <c r="T12" s="78" t="n"/>
+      <c r="U12" s="85" t="n"/>
+      <c r="V12" s="86" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="60" t="n"/>
-      <c r="C13" s="61" t="n"/>
-      <c r="D13" s="62" t="n"/>
-      <c r="E13" s="79" t="inlineStr">
+      <c r="B13" s="66" t="n"/>
+      <c r="C13" s="67" t="n"/>
+      <c r="D13" s="68" t="n"/>
+      <c r="E13" s="69" t="n"/>
+      <c r="F13" s="70" t="n"/>
+      <c r="G13" s="87" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F13" s="80" t="inlineStr">
+      <c r="H13" s="88" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
-      <c r="G13" s="81" t="n"/>
-      <c r="H13" s="82" t="n"/>
-      <c r="I13" s="83" t="inlineStr">
+      <c r="I13" s="89" t="n"/>
+      <c r="J13" s="90" t="n"/>
+      <c r="K13" s="91" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
-      <c r="J13" s="84" t="inlineStr">
+      <c r="L13" s="92" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K13" s="69" t="n"/>
-      <c r="L13" s="70" t="n"/>
-      <c r="M13" s="71" t="n"/>
-      <c r="N13" s="72" t="n"/>
-      <c r="O13" s="85" t="n"/>
-      <c r="P13" s="86" t="n"/>
-      <c r="Q13" s="87" t="n"/>
-      <c r="R13" s="88" t="n"/>
-      <c r="S13" s="77" t="n"/>
-      <c r="T13" s="78" t="n"/>
+      <c r="M13" s="77" t="n"/>
+      <c r="N13" s="78" t="n"/>
+      <c r="O13" s="79" t="n"/>
+      <c r="P13" s="80" t="n"/>
+      <c r="Q13" s="93" t="n"/>
+      <c r="R13" s="94" t="n"/>
+      <c r="S13" s="95" t="n"/>
+      <c r="T13" s="96" t="n"/>
+      <c r="U13" s="85" t="n"/>
+      <c r="V13" s="86" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="60" t="n"/>
-      <c r="C14" s="61" t="n"/>
-      <c r="D14" s="62" t="n"/>
-      <c r="E14" s="63" t="n"/>
-      <c r="F14" s="64" t="n"/>
-      <c r="G14" s="81" t="n"/>
-      <c r="H14" s="82" t="n"/>
-      <c r="I14" s="83" t="inlineStr">
+      <c r="B14" s="66" t="n"/>
+      <c r="C14" s="67" t="n"/>
+      <c r="D14" s="68" t="n"/>
+      <c r="E14" s="69" t="n"/>
+      <c r="F14" s="70" t="n"/>
+      <c r="G14" s="71" t="n"/>
+      <c r="H14" s="72" t="n"/>
+      <c r="I14" s="89" t="n"/>
+      <c r="J14" s="90" t="n"/>
+      <c r="K14" s="91" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="J14" s="84" t="inlineStr">
+      <c r="L14" s="92" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
-      <c r="K14" s="69" t="n"/>
-      <c r="L14" s="70" t="n"/>
-      <c r="M14" s="71" t="n"/>
-      <c r="N14" s="72" t="n"/>
-      <c r="O14" s="73" t="inlineStr">
+      <c r="M14" s="77" t="n"/>
+      <c r="N14" s="78" t="n"/>
+      <c r="O14" s="79" t="n"/>
+      <c r="P14" s="80" t="n"/>
+      <c r="Q14" s="81" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="P14" s="74" t="inlineStr">
+      <c r="R14" s="82" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
-      <c r="Q14" s="75" t="inlineStr">
+      <c r="S14" s="83" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="R14" s="76" t="inlineStr">
+      <c r="T14" s="84" t="inlineStr">
         <is>
           <t>15.23</t>
         </is>
       </c>
-      <c r="S14" s="77" t="n"/>
-      <c r="T14" s="78" t="n"/>
+      <c r="U14" s="85" t="n"/>
+      <c r="V14" s="86" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="60" t="n"/>
-      <c r="C15" s="61" t="n"/>
-      <c r="D15" s="62" t="n"/>
-      <c r="E15" s="79" t="inlineStr">
+      <c r="B15" s="66" t="n"/>
+      <c r="C15" s="67" t="n"/>
+      <c r="D15" s="68" t="n"/>
+      <c r="E15" s="69" t="n"/>
+      <c r="F15" s="70" t="n"/>
+      <c r="G15" s="87" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F15" s="80" t="inlineStr">
+      <c r="H15" s="88" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
-      <c r="G15" s="81" t="n"/>
-      <c r="H15" s="82" t="n"/>
-      <c r="I15" s="83" t="inlineStr">
+      <c r="I15" s="89" t="n"/>
+      <c r="J15" s="90" t="n"/>
+      <c r="K15" s="91" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
-      <c r="J15" s="84" t="inlineStr">
+      <c r="L15" s="92" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K15" s="69" t="n"/>
-      <c r="L15" s="70" t="n"/>
-      <c r="M15" s="71" t="n"/>
-      <c r="N15" s="72" t="n"/>
-      <c r="O15" s="85" t="n"/>
-      <c r="P15" s="86" t="n"/>
-      <c r="Q15" s="87" t="n"/>
-      <c r="R15" s="88" t="n"/>
-      <c r="S15" s="77" t="n"/>
-      <c r="T15" s="78" t="n"/>
+      <c r="M15" s="77" t="n"/>
+      <c r="N15" s="78" t="n"/>
+      <c r="O15" s="79" t="n"/>
+      <c r="P15" s="80" t="n"/>
+      <c r="Q15" s="93" t="n"/>
+      <c r="R15" s="94" t="n"/>
+      <c r="S15" s="95" t="n"/>
+      <c r="T15" s="96" t="n"/>
+      <c r="U15" s="85" t="n"/>
+      <c r="V15" s="86" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="91" t="n"/>
-      <c r="C16" s="92" t="n"/>
-      <c r="D16" s="93" t="n"/>
-      <c r="E16" s="94" t="n"/>
-      <c r="F16" s="95" t="n"/>
-      <c r="G16" s="96" t="n"/>
-      <c r="H16" s="97" t="n"/>
-      <c r="I16" s="98" t="inlineStr">
+      <c r="B16" s="99" t="n"/>
+      <c r="C16" s="100" t="n"/>
+      <c r="D16" s="101" t="n"/>
+      <c r="E16" s="102" t="n"/>
+      <c r="F16" s="103" t="n"/>
+      <c r="G16" s="104" t="n"/>
+      <c r="H16" s="105" t="n"/>
+      <c r="I16" s="106" t="n"/>
+      <c r="J16" s="107" t="n"/>
+      <c r="K16" s="108" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="J16" s="99" t="inlineStr">
+      <c r="L16" s="109" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
-      <c r="K16" s="100" t="n"/>
-      <c r="L16" s="101" t="n"/>
-      <c r="M16" s="102" t="n"/>
-      <c r="N16" s="103" t="n"/>
-      <c r="O16" s="104" t="inlineStr">
+      <c r="M16" s="110" t="n"/>
+      <c r="N16" s="111" t="n"/>
+      <c r="O16" s="112" t="n"/>
+      <c r="P16" s="113" t="n"/>
+      <c r="Q16" s="114" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="P16" s="105" t="inlineStr">
+      <c r="R16" s="115" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
-      <c r="Q16" s="106" t="inlineStr">
+      <c r="S16" s="116" t="inlineStr">
         <is>
           <t>gundam</t>
         </is>
       </c>
-      <c r="R16" s="107" t="inlineStr">
+      <c r="T16" s="117" t="inlineStr">
         <is>
           <t>12.57</t>
         </is>
       </c>
-      <c r="S16" s="108" t="n"/>
-      <c r="T16" s="109" t="n"/>
+      <c r="U16" s="118" t="n"/>
+      <c r="V16" s="119" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="110" t="inlineStr">
+      <c r="B17" s="120" t="inlineStr">
         <is>
           <t>sum</t>
         </is>
       </c>
-      <c r="C17" s="111" t="n">
+      <c r="C17" s="121" t="n">
         <v>70</v>
       </c>
-      <c r="D17" s="112" t="n"/>
-      <c r="E17" s="113" t="n">
+      <c r="D17" s="122" t="n"/>
+      <c r="E17" s="123" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="124" t="n"/>
+      <c r="G17" s="125" t="n">
         <v>14944.22</v>
       </c>
-      <c r="F17" s="114" t="n"/>
-      <c r="G17" s="115" t="n">
+      <c r="H17" s="126" t="n"/>
+      <c r="I17" s="127" t="n">
         <v>68</v>
       </c>
-      <c r="H17" s="116" t="n"/>
-      <c r="I17" s="117" t="n">
+      <c r="J17" s="128" t="n"/>
+      <c r="K17" s="129" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="118" t="n"/>
-      <c r="K17" s="119" t="n">
+      <c r="L17" s="130" t="n"/>
+      <c r="M17" s="131" t="n">
         <v>0</v>
       </c>
-      <c r="L17" s="120" t="n"/>
-      <c r="M17" s="121" t="n">
+      <c r="N17" s="132" t="n"/>
+      <c r="O17" s="133" t="n">
         <v>0</v>
       </c>
-      <c r="N17" s="122" t="n"/>
-      <c r="O17" s="123" t="n">
+      <c r="P17" s="134" t="n"/>
+      <c r="Q17" s="135" t="n">
         <v>0</v>
       </c>
-      <c r="P17" s="124" t="n">
+      <c r="R17" s="136" t="n">
         <v>343.7</v>
       </c>
-      <c r="Q17" s="125" t="n">
+      <c r="S17" s="137" t="n">
         <v>0</v>
       </c>
-      <c r="R17" s="126" t="n">
+      <c r="T17" s="138" t="n">
         <v>343.7</v>
       </c>
-      <c r="S17" s="127" t="n">
+      <c r="U17" s="139" t="n">
         <v>15082.22</v>
       </c>
-      <c r="T17" s="128" t="inlineStr">
+      <c r="V17" s="140" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="129" t="inlineStr">
+      <c r="B18" s="141" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="C18" s="130" t="n"/>
-      <c r="D18" s="131" t="n"/>
-      <c r="E18" s="132" t="n"/>
-      <c r="F18" s="133" t="n"/>
-      <c r="G18" s="134" t="n"/>
-      <c r="H18" s="135" t="n"/>
-      <c r="I18" s="136" t="n"/>
-      <c r="J18" s="137" t="n"/>
-      <c r="K18" s="138" t="n"/>
-      <c r="L18" s="139" t="n"/>
-      <c r="M18" s="140" t="n"/>
-      <c r="N18" s="141" t="n"/>
-      <c r="O18" s="142" t="n">
+      <c r="C18" s="142" t="n"/>
+      <c r="D18" s="143" t="n"/>
+      <c r="E18" s="144" t="n"/>
+      <c r="F18" s="145" t="n"/>
+      <c r="G18" s="146" t="n"/>
+      <c r="H18" s="147" t="n"/>
+      <c r="I18" s="148" t="n"/>
+      <c r="J18" s="149" t="n"/>
+      <c r="K18" s="150" t="n"/>
+      <c r="L18" s="151" t="n"/>
+      <c r="M18" s="152" t="n"/>
+      <c r="N18" s="153" t="n"/>
+      <c r="O18" s="154" t="n"/>
+      <c r="P18" s="155" t="n"/>
+      <c r="Q18" s="156" t="n">
         <v>0</v>
       </c>
-      <c r="P18" s="143" t="n">
+      <c r="R18" s="157" t="n">
         <v>343.7</v>
       </c>
-      <c r="Q18" s="144" t="n">
+      <c r="S18" s="158" t="n">
         <v>0</v>
       </c>
-      <c r="R18" s="145" t="n">
+      <c r="T18" s="159" t="n">
         <v>343.7</v>
       </c>
-      <c r="S18" s="146" t="n"/>
-      <c r="T18" s="147" t="n"/>
+      <c r="U18" s="160" t="n"/>
+      <c r="V18" s="161" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="41" t="inlineStr">
+      <c r="B19" s="45" t="inlineStr">
         <is>
           <t>02/01/2026</t>
         </is>
       </c>
-      <c r="C19" s="42" t="n"/>
-      <c r="D19" s="43" t="n"/>
-      <c r="E19" s="148" t="inlineStr">
+      <c r="C19" s="46" t="n"/>
+      <c r="D19" s="47" t="n"/>
+      <c r="E19" s="48" t="n"/>
+      <c r="F19" s="49" t="n"/>
+      <c r="G19" s="162" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
-      <c r="F19" s="149" t="inlineStr">
+      <c r="H19" s="163" t="inlineStr">
         <is>
           <t>2993</t>
         </is>
       </c>
-      <c r="G19" s="150" t="n"/>
-      <c r="H19" s="151" t="n"/>
-      <c r="I19" s="48" t="n"/>
-      <c r="J19" s="49" t="n"/>
-      <c r="K19" s="50" t="n"/>
-      <c r="L19" s="51" t="n"/>
-      <c r="M19" s="52" t="n"/>
-      <c r="N19" s="53" t="n"/>
-      <c r="O19" s="152" t="n"/>
-      <c r="P19" s="153" t="n"/>
-      <c r="Q19" s="56" t="inlineStr">
+      <c r="I19" s="164" t="n"/>
+      <c r="J19" s="165" t="n"/>
+      <c r="K19" s="54" t="n"/>
+      <c r="L19" s="55" t="n"/>
+      <c r="M19" s="56" t="n"/>
+      <c r="N19" s="57" t="n"/>
+      <c r="O19" s="58" t="n"/>
+      <c r="P19" s="59" t="n"/>
+      <c r="Q19" s="166" t="n"/>
+      <c r="R19" s="167" t="n"/>
+      <c r="S19" s="62" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
-      <c r="R19" s="57" t="inlineStr">
+      <c r="T19" s="63" t="inlineStr">
         <is>
           <t>2993</t>
         </is>
       </c>
-      <c r="S19" s="58" t="n"/>
-      <c r="T19" s="59" t="n"/>
+      <c r="U19" s="64" t="n"/>
+      <c r="V19" s="65" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="60" t="n"/>
-      <c r="C20" s="61" t="n"/>
-      <c r="D20" s="62" t="n"/>
-      <c r="E20" s="79" t="inlineStr">
+      <c r="B20" s="66" t="n"/>
+      <c r="C20" s="67" t="n"/>
+      <c r="D20" s="68" t="n"/>
+      <c r="E20" s="69" t="n"/>
+      <c r="F20" s="70" t="n"/>
+      <c r="G20" s="87" t="inlineStr">
         <is>
           <t>7000</t>
         </is>
       </c>
-      <c r="F20" s="80" t="inlineStr">
+      <c r="H20" s="88" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
-      <c r="G20" s="81" t="n"/>
-      <c r="H20" s="82" t="n"/>
-      <c r="I20" s="67" t="n"/>
-      <c r="J20" s="68" t="n"/>
-      <c r="K20" s="69" t="n"/>
-      <c r="L20" s="70" t="n"/>
-      <c r="M20" s="71" t="n"/>
-      <c r="N20" s="72" t="n"/>
-      <c r="O20" s="85" t="n"/>
-      <c r="P20" s="86" t="n"/>
-      <c r="Q20" s="75" t="inlineStr">
+      <c r="I20" s="89" t="n"/>
+      <c r="J20" s="90" t="n"/>
+      <c r="K20" s="75" t="n"/>
+      <c r="L20" s="76" t="n"/>
+      <c r="M20" s="77" t="n"/>
+      <c r="N20" s="78" t="n"/>
+      <c r="O20" s="79" t="n"/>
+      <c r="P20" s="80" t="n"/>
+      <c r="Q20" s="93" t="n"/>
+      <c r="R20" s="94" t="n"/>
+      <c r="S20" s="83" t="inlineStr">
         <is>
           <t>7000</t>
         </is>
       </c>
-      <c r="R20" s="76" t="inlineStr">
+      <c r="T20" s="84" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
-      <c r="S20" s="77" t="n"/>
-      <c r="T20" s="78" t="n"/>
+      <c r="U20" s="85" t="n"/>
+      <c r="V20" s="86" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="60" t="n"/>
-      <c r="C21" s="61" t="n"/>
-      <c r="D21" s="62" t="n"/>
-      <c r="E21" s="63" t="n"/>
-      <c r="F21" s="64" t="n"/>
-      <c r="G21" s="65" t="inlineStr">
+      <c r="B21" s="66" t="n"/>
+      <c r="C21" s="67" t="n"/>
+      <c r="D21" s="68" t="n"/>
+      <c r="E21" s="69" t="n"/>
+      <c r="F21" s="70" t="n"/>
+      <c r="G21" s="71" t="n"/>
+      <c r="H21" s="72" t="n"/>
+      <c r="I21" s="73" t="inlineStr">
         <is>
           <t>LRT</t>
         </is>
       </c>
-      <c r="H21" s="66" t="inlineStr">
+      <c r="J21" s="74" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="I21" s="67" t="n"/>
-      <c r="J21" s="68" t="n"/>
-      <c r="K21" s="69" t="n"/>
-      <c r="L21" s="70" t="n"/>
-      <c r="M21" s="71" t="n"/>
-      <c r="N21" s="72" t="n"/>
-      <c r="O21" s="73" t="inlineStr">
+      <c r="K21" s="75" t="n"/>
+      <c r="L21" s="76" t="n"/>
+      <c r="M21" s="77" t="n"/>
+      <c r="N21" s="78" t="n"/>
+      <c r="O21" s="79" t="n"/>
+      <c r="P21" s="80" t="n"/>
+      <c r="Q21" s="81" t="inlineStr">
         <is>
           <t>LRT</t>
         </is>
       </c>
-      <c r="P21" s="74" t="inlineStr">
+      <c r="R21" s="82" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="Q21" s="75" t="inlineStr">
+      <c r="S21" s="83" t="inlineStr">
         <is>
           <t>LRT</t>
         </is>
       </c>
-      <c r="R21" s="76" t="inlineStr">
+      <c r="T21" s="84" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="S21" s="77" t="n"/>
-      <c r="T21" s="78" t="n"/>
+      <c r="U21" s="85" t="n"/>
+      <c r="V21" s="86" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="60" t="n"/>
-      <c r="C22" s="61" t="n"/>
-      <c r="D22" s="62" t="n"/>
-      <c r="E22" s="63" t="n"/>
-      <c r="F22" s="64" t="n"/>
-      <c r="G22" s="65" t="inlineStr">
+      <c r="B22" s="66" t="n"/>
+      <c r="C22" s="67" t="n"/>
+      <c r="D22" s="68" t="n"/>
+      <c r="E22" s="69" t="n"/>
+      <c r="F22" s="70" t="n"/>
+      <c r="G22" s="71" t="n"/>
+      <c r="H22" s="72" t="n"/>
+      <c r="I22" s="73" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="H22" s="66" t="inlineStr">
+      <c r="J22" s="74" t="inlineStr">
         <is>
           <t>10.8</t>
         </is>
       </c>
-      <c r="I22" s="67" t="n"/>
-      <c r="J22" s="68" t="n"/>
-      <c r="K22" s="69" t="n"/>
-      <c r="L22" s="70" t="n"/>
-      <c r="M22" s="71" t="n"/>
-      <c r="N22" s="72" t="n"/>
-      <c r="O22" s="73" t="inlineStr">
+      <c r="K22" s="75" t="n"/>
+      <c r="L22" s="76" t="n"/>
+      <c r="M22" s="77" t="n"/>
+      <c r="N22" s="78" t="n"/>
+      <c r="O22" s="79" t="n"/>
+      <c r="P22" s="80" t="n"/>
+      <c r="Q22" s="81" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="P22" s="74" t="inlineStr">
+      <c r="R22" s="82" t="inlineStr">
         <is>
           <t>10.8</t>
         </is>
       </c>
-      <c r="Q22" s="75" t="inlineStr">
+      <c r="S22" s="83" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="R22" s="76" t="inlineStr">
+      <c r="T22" s="84" t="inlineStr">
         <is>
           <t>10.8</t>
         </is>
       </c>
-      <c r="S22" s="77" t="n"/>
-      <c r="T22" s="78" t="n"/>
+      <c r="U22" s="85" t="n"/>
+      <c r="V22" s="86" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="60" t="n"/>
-      <c r="C23" s="61" t="n"/>
-      <c r="D23" s="62" t="n"/>
-      <c r="E23" s="63" t="n"/>
-      <c r="F23" s="64" t="n"/>
-      <c r="G23" s="65" t="inlineStr">
+      <c r="B23" s="66" t="n"/>
+      <c r="C23" s="67" t="n"/>
+      <c r="D23" s="68" t="n"/>
+      <c r="E23" s="69" t="n"/>
+      <c r="F23" s="70" t="n"/>
+      <c r="G23" s="71" t="n"/>
+      <c r="H23" s="72" t="n"/>
+      <c r="I23" s="73" t="inlineStr">
         <is>
           <t>MTR</t>
         </is>
       </c>
-      <c r="H23" s="66" t="inlineStr">
+      <c r="J23" s="74" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="I23" s="67" t="n"/>
-      <c r="J23" s="68" t="n"/>
-      <c r="K23" s="69" t="n"/>
-      <c r="L23" s="70" t="n"/>
-      <c r="M23" s="71" t="n"/>
-      <c r="N23" s="72" t="n"/>
-      <c r="O23" s="73" t="inlineStr">
+      <c r="K23" s="75" t="n"/>
+      <c r="L23" s="76" t="n"/>
+      <c r="M23" s="77" t="n"/>
+      <c r="N23" s="78" t="n"/>
+      <c r="O23" s="79" t="n"/>
+      <c r="P23" s="80" t="n"/>
+      <c r="Q23" s="81" t="inlineStr">
         <is>
           <t>MTR</t>
         </is>
       </c>
-      <c r="P23" s="74" t="inlineStr">
+      <c r="R23" s="82" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="Q23" s="75" t="inlineStr">
+      <c r="S23" s="83" t="inlineStr">
         <is>
           <t>MTR</t>
         </is>
       </c>
-      <c r="R23" s="76" t="inlineStr">
+      <c r="T23" s="84" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="S23" s="77" t="n"/>
-      <c r="T23" s="78" t="n"/>
+      <c r="U23" s="85" t="n"/>
+      <c r="V23" s="86" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="60" t="n"/>
-      <c r="C24" s="61" t="n"/>
-      <c r="D24" s="62" t="n"/>
-      <c r="E24" s="63" t="n"/>
-      <c r="F24" s="64" t="n"/>
-      <c r="G24" s="65" t="inlineStr">
+      <c r="B24" s="66" t="n"/>
+      <c r="C24" s="67" t="n"/>
+      <c r="D24" s="68" t="n"/>
+      <c r="E24" s="69" t="n"/>
+      <c r="F24" s="70" t="n"/>
+      <c r="G24" s="71" t="n"/>
+      <c r="H24" s="72" t="n"/>
+      <c r="I24" s="73" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="H24" s="66" t="inlineStr">
+      <c r="J24" s="74" t="inlineStr">
         <is>
           <t>10.4</t>
         </is>
       </c>
-      <c r="I24" s="67" t="n"/>
-      <c r="J24" s="68" t="n"/>
-      <c r="K24" s="69" t="n"/>
-      <c r="L24" s="70" t="n"/>
-      <c r="M24" s="71" t="n"/>
-      <c r="N24" s="72" t="n"/>
-      <c r="O24" s="73" t="inlineStr">
+      <c r="K24" s="75" t="n"/>
+      <c r="L24" s="76" t="n"/>
+      <c r="M24" s="77" t="n"/>
+      <c r="N24" s="78" t="n"/>
+      <c r="O24" s="79" t="n"/>
+      <c r="P24" s="80" t="n"/>
+      <c r="Q24" s="81" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="P24" s="74" t="inlineStr">
+      <c r="R24" s="82" t="inlineStr">
         <is>
           <t>10.4</t>
         </is>
       </c>
-      <c r="Q24" s="75" t="inlineStr">
+      <c r="S24" s="83" t="inlineStr">
         <is>
           <t>Bus</t>
         </is>
       </c>
-      <c r="R24" s="76" t="inlineStr">
+      <c r="T24" s="84" t="inlineStr">
         <is>
           <t>10.4</t>
         </is>
       </c>
-      <c r="S24" s="77" t="n"/>
-      <c r="T24" s="78" t="n"/>
+      <c r="U24" s="85" t="n"/>
+      <c r="V24" s="86" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="60" t="n"/>
-      <c r="C25" s="61" t="n"/>
-      <c r="D25" s="62" t="n"/>
-      <c r="E25" s="79" t="inlineStr">
+      <c r="B25" s="66" t="n"/>
+      <c r="C25" s="67" t="n"/>
+      <c r="D25" s="68" t="n"/>
+      <c r="E25" s="69" t="n"/>
+      <c r="F25" s="70" t="n"/>
+      <c r="G25" s="87" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F25" s="80" t="inlineStr">
+      <c r="H25" s="88" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
-      <c r="G25" s="81" t="n"/>
-      <c r="H25" s="82" t="n"/>
-      <c r="I25" s="83" t="inlineStr">
+      <c r="I25" s="89" t="n"/>
+      <c r="J25" s="90" t="n"/>
+      <c r="K25" s="91" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
-      <c r="J25" s="84" t="inlineStr">
+      <c r="L25" s="92" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K25" s="69" t="n"/>
-      <c r="L25" s="70" t="n"/>
-      <c r="M25" s="71" t="n"/>
-      <c r="N25" s="72" t="n"/>
-      <c r="O25" s="85" t="n"/>
-      <c r="P25" s="86" t="n"/>
-      <c r="Q25" s="87" t="n"/>
-      <c r="R25" s="88" t="n"/>
-      <c r="S25" s="77" t="n"/>
-      <c r="T25" s="78" t="n"/>
+      <c r="M25" s="77" t="n"/>
+      <c r="N25" s="78" t="n"/>
+      <c r="O25" s="79" t="n"/>
+      <c r="P25" s="80" t="n"/>
+      <c r="Q25" s="93" t="n"/>
+      <c r="R25" s="94" t="n"/>
+      <c r="S25" s="95" t="n"/>
+      <c r="T25" s="96" t="n"/>
+      <c r="U25" s="85" t="n"/>
+      <c r="V25" s="86" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="60" t="n"/>
-      <c r="C26" s="61" t="n"/>
-      <c r="D26" s="62" t="n"/>
-      <c r="E26" s="63" t="n"/>
-      <c r="F26" s="64" t="n"/>
-      <c r="G26" s="81" t="n"/>
-      <c r="H26" s="82" t="n"/>
-      <c r="I26" s="83" t="inlineStr">
+      <c r="B26" s="66" t="n"/>
+      <c r="C26" s="67" t="n"/>
+      <c r="D26" s="68" t="n"/>
+      <c r="E26" s="69" t="n"/>
+      <c r="F26" s="70" t="n"/>
+      <c r="G26" s="71" t="n"/>
+      <c r="H26" s="72" t="n"/>
+      <c r="I26" s="89" t="n"/>
+      <c r="J26" s="90" t="n"/>
+      <c r="K26" s="91" t="inlineStr">
         <is>
           <t>Piggy</t>
         </is>
       </c>
-      <c r="J26" s="84" t="inlineStr">
+      <c r="L26" s="92" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
-      <c r="K26" s="69" t="n"/>
-      <c r="L26" s="70" t="n"/>
-      <c r="M26" s="71" t="n"/>
-      <c r="N26" s="72" t="n"/>
-      <c r="O26" s="73" t="inlineStr">
+      <c r="M26" s="77" t="n"/>
+      <c r="N26" s="78" t="n"/>
+      <c r="O26" s="79" t="n"/>
+      <c r="P26" s="80" t="n"/>
+      <c r="Q26" s="81" t="inlineStr">
         <is>
           <t>Piggy</t>
         </is>
       </c>
-      <c r="P26" s="74" t="inlineStr">
+      <c r="R26" s="82" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
-      <c r="Q26" s="75" t="inlineStr">
+      <c r="S26" s="83" t="inlineStr">
         <is>
           <t>Piggy</t>
         </is>
       </c>
-      <c r="R26" s="76" t="inlineStr">
+      <c r="T26" s="84" t="inlineStr">
         <is>
           <t>2520</t>
         </is>
       </c>
-      <c r="S26" s="77" t="n"/>
-      <c r="T26" s="78" t="n"/>
+      <c r="U26" s="85" t="n"/>
+      <c r="V26" s="86" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="60" t="n"/>
-      <c r="C27" s="61" t="n"/>
-      <c r="D27" s="62" t="n"/>
-      <c r="E27" s="79" t="inlineStr">
+      <c r="B27" s="66" t="n"/>
+      <c r="C27" s="67" t="n"/>
+      <c r="D27" s="68" t="n"/>
+      <c r="E27" s="69" t="n"/>
+      <c r="F27" s="70" t="n"/>
+      <c r="G27" s="87" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F27" s="80" t="inlineStr">
+      <c r="H27" s="88" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="G27" s="81" t="n"/>
-      <c r="H27" s="82" t="n"/>
-      <c r="I27" s="83" t="inlineStr">
+      <c r="I27" s="89" t="n"/>
+      <c r="J27" s="90" t="n"/>
+      <c r="K27" s="91" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="J27" s="84" t="inlineStr">
+      <c r="L27" s="92" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K27" s="69" t="n"/>
-      <c r="L27" s="70" t="n"/>
-      <c r="M27" s="71" t="n"/>
-      <c r="N27" s="72" t="n"/>
-      <c r="O27" s="85" t="n"/>
-      <c r="P27" s="86" t="n"/>
-      <c r="Q27" s="87" t="n"/>
-      <c r="R27" s="88" t="n"/>
-      <c r="S27" s="77" t="n"/>
-      <c r="T27" s="78" t="n"/>
+      <c r="M27" s="77" t="n"/>
+      <c r="N27" s="78" t="n"/>
+      <c r="O27" s="79" t="n"/>
+      <c r="P27" s="80" t="n"/>
+      <c r="Q27" s="93" t="n"/>
+      <c r="R27" s="94" t="n"/>
+      <c r="S27" s="95" t="n"/>
+      <c r="T27" s="96" t="n"/>
+      <c r="U27" s="85" t="n"/>
+      <c r="V27" s="86" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="60" t="n"/>
-      <c r="C28" s="61" t="n"/>
-      <c r="D28" s="62" t="n"/>
-      <c r="E28" s="63" t="n"/>
-      <c r="F28" s="64" t="n"/>
-      <c r="G28" s="81" t="n"/>
-      <c r="H28" s="82" t="n"/>
-      <c r="I28" s="83" t="inlineStr">
+      <c r="B28" s="66" t="n"/>
+      <c r="C28" s="67" t="n"/>
+      <c r="D28" s="68" t="n"/>
+      <c r="E28" s="69" t="n"/>
+      <c r="F28" s="70" t="n"/>
+      <c r="G28" s="71" t="n"/>
+      <c r="H28" s="72" t="n"/>
+      <c r="I28" s="89" t="n"/>
+      <c r="J28" s="90" t="n"/>
+      <c r="K28" s="91" t="inlineStr">
         <is>
           <t>Piggy play</t>
         </is>
       </c>
-      <c r="J28" s="84" t="inlineStr">
+      <c r="L28" s="92" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="K28" s="69" t="n"/>
-      <c r="L28" s="70" t="n"/>
-      <c r="M28" s="71" t="n"/>
-      <c r="N28" s="72" t="n"/>
-      <c r="O28" s="73" t="inlineStr">
+      <c r="M28" s="77" t="n"/>
+      <c r="N28" s="78" t="n"/>
+      <c r="O28" s="79" t="n"/>
+      <c r="P28" s="80" t="n"/>
+      <c r="Q28" s="81" t="inlineStr">
         <is>
           <t>Piggy play</t>
         </is>
       </c>
-      <c r="P28" s="74" t="inlineStr">
+      <c r="R28" s="82" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="Q28" s="75" t="inlineStr">
+      <c r="S28" s="83" t="inlineStr">
         <is>
           <t>Piggy play</t>
         </is>
       </c>
-      <c r="R28" s="76" t="inlineStr">
+      <c r="T28" s="84" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="S28" s="77" t="n"/>
-      <c r="T28" s="78" t="n"/>
+      <c r="U28" s="85" t="n"/>
+      <c r="V28" s="86" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="60" t="n"/>
-      <c r="C29" s="61" t="n"/>
-      <c r="D29" s="62" t="n"/>
-      <c r="E29" s="79" t="inlineStr">
+      <c r="B29" s="66" t="n"/>
+      <c r="C29" s="67" t="n"/>
+      <c r="D29" s="68" t="n"/>
+      <c r="E29" s="69" t="n"/>
+      <c r="F29" s="70" t="n"/>
+      <c r="G29" s="87" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F29" s="80" t="inlineStr">
+      <c r="H29" s="88" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="G29" s="81" t="n"/>
-      <c r="H29" s="82" t="n"/>
-      <c r="I29" s="83" t="inlineStr">
+      <c r="I29" s="89" t="n"/>
+      <c r="J29" s="90" t="n"/>
+      <c r="K29" s="91" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="J29" s="84" t="inlineStr">
+      <c r="L29" s="92" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K29" s="69" t="n"/>
-      <c r="L29" s="70" t="n"/>
-      <c r="M29" s="71" t="n"/>
-      <c r="N29" s="72" t="n"/>
-      <c r="O29" s="85" t="n"/>
-      <c r="P29" s="86" t="n"/>
-      <c r="Q29" s="87" t="n"/>
-      <c r="R29" s="88" t="n"/>
-      <c r="S29" s="77" t="n"/>
-      <c r="T29" s="78" t="n"/>
+      <c r="M29" s="77" t="n"/>
+      <c r="N29" s="78" t="n"/>
+      <c r="O29" s="79" t="n"/>
+      <c r="P29" s="80" t="n"/>
+      <c r="Q29" s="93" t="n"/>
+      <c r="R29" s="94" t="n"/>
+      <c r="S29" s="95" t="n"/>
+      <c r="T29" s="96" t="n"/>
+      <c r="U29" s="85" t="n"/>
+      <c r="V29" s="86" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="60" t="n"/>
-      <c r="C30" s="61" t="n"/>
-      <c r="D30" s="62" t="n"/>
-      <c r="E30" s="63" t="n"/>
-      <c r="F30" s="64" t="n"/>
-      <c r="G30" s="81" t="n"/>
-      <c r="H30" s="82" t="n"/>
-      <c r="I30" s="83" t="inlineStr">
+      <c r="B30" s="66" t="n"/>
+      <c r="C30" s="67" t="n"/>
+      <c r="D30" s="68" t="n"/>
+      <c r="E30" s="69" t="n"/>
+      <c r="F30" s="70" t="n"/>
+      <c r="G30" s="71" t="n"/>
+      <c r="H30" s="72" t="n"/>
+      <c r="I30" s="89" t="n"/>
+      <c r="J30" s="90" t="n"/>
+      <c r="K30" s="91" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="J30" s="84" t="inlineStr">
+      <c r="L30" s="92" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="K30" s="69" t="n"/>
-      <c r="L30" s="70" t="n"/>
-      <c r="M30" s="71" t="n"/>
-      <c r="N30" s="72" t="n"/>
-      <c r="O30" s="73" t="inlineStr">
+      <c r="M30" s="77" t="n"/>
+      <c r="N30" s="78" t="n"/>
+      <c r="O30" s="79" t="n"/>
+      <c r="P30" s="80" t="n"/>
+      <c r="Q30" s="81" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="P30" s="74" t="inlineStr">
+      <c r="R30" s="82" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="Q30" s="75" t="inlineStr">
+      <c r="S30" s="83" t="inlineStr">
         <is>
           <t>Drink</t>
         </is>
       </c>
-      <c r="R30" s="76" t="inlineStr">
+      <c r="T30" s="84" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="S30" s="77" t="n"/>
-      <c r="T30" s="78" t="n"/>
+      <c r="U30" s="85" t="n"/>
+      <c r="V30" s="86" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="60" t="n"/>
-      <c r="C31" s="61" t="n"/>
-      <c r="D31" s="62" t="n"/>
-      <c r="E31" s="79" t="inlineStr">
+      <c r="B31" s="66" t="n"/>
+      <c r="C31" s="67" t="n"/>
+      <c r="D31" s="68" t="n"/>
+      <c r="E31" s="69" t="n"/>
+      <c r="F31" s="70" t="n"/>
+      <c r="G31" s="87" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="F31" s="80" t="inlineStr">
+      <c r="H31" s="88" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
-      <c r="G31" s="81" t="n"/>
-      <c r="H31" s="82" t="n"/>
-      <c r="I31" s="83" t="inlineStr">
+      <c r="I31" s="89" t="n"/>
+      <c r="J31" s="90" t="n"/>
+      <c r="K31" s="91" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
-      <c r="J31" s="84" t="inlineStr">
+      <c r="L31" s="92" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K31" s="69" t="n"/>
-      <c r="L31" s="70" t="n"/>
-      <c r="M31" s="71" t="n"/>
-      <c r="N31" s="72" t="n"/>
-      <c r="O31" s="85" t="n"/>
-      <c r="P31" s="86" t="n"/>
-      <c r="Q31" s="87" t="n"/>
-      <c r="R31" s="88" t="n"/>
-      <c r="S31" s="77" t="n"/>
-      <c r="T31" s="78" t="n"/>
+      <c r="M31" s="77" t="n"/>
+      <c r="N31" s="78" t="n"/>
+      <c r="O31" s="79" t="n"/>
+      <c r="P31" s="80" t="n"/>
+      <c r="Q31" s="93" t="n"/>
+      <c r="R31" s="94" t="n"/>
+      <c r="S31" s="95" t="n"/>
+      <c r="T31" s="96" t="n"/>
+      <c r="U31" s="85" t="n"/>
+      <c r="V31" s="86" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="60" t="n"/>
-      <c r="C32" s="61" t="n"/>
-      <c r="D32" s="62" t="n"/>
-      <c r="E32" s="63" t="n"/>
-      <c r="F32" s="64" t="n"/>
-      <c r="G32" s="81" t="n"/>
-      <c r="H32" s="82" t="n"/>
-      <c r="I32" s="83" t="inlineStr">
+      <c r="B32" s="66" t="n"/>
+      <c r="C32" s="67" t="n"/>
+      <c r="D32" s="68" t="n"/>
+      <c r="E32" s="69" t="n"/>
+      <c r="F32" s="70" t="n"/>
+      <c r="G32" s="71" t="n"/>
+      <c r="H32" s="72" t="n"/>
+      <c r="I32" s="89" t="n"/>
+      <c r="J32" s="90" t="n"/>
+      <c r="K32" s="91" t="inlineStr">
         <is>
           <t>Dinner</t>
         </is>
       </c>
-      <c r="J32" s="84" t="inlineStr">
+      <c r="L32" s="92" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
-      <c r="K32" s="69" t="n"/>
-      <c r="L32" s="70" t="n"/>
-      <c r="M32" s="71" t="n"/>
-      <c r="N32" s="72" t="n"/>
-      <c r="O32" s="73" t="inlineStr">
+      <c r="M32" s="77" t="n"/>
+      <c r="N32" s="78" t="n"/>
+      <c r="O32" s="79" t="n"/>
+      <c r="P32" s="80" t="n"/>
+      <c r="Q32" s="81" t="inlineStr">
         <is>
           <t>Dinner</t>
         </is>
       </c>
-      <c r="P32" s="74" t="inlineStr">
+      <c r="R32" s="82" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
-      <c r="Q32" s="75" t="inlineStr">
+      <c r="S32" s="83" t="inlineStr">
         <is>
           <t>Dinner</t>
         </is>
       </c>
-      <c r="R32" s="76" t="inlineStr">
+      <c r="T32" s="84" t="inlineStr">
         <is>
           <t>231.6</t>
         </is>
       </c>
-      <c r="S32" s="77" t="n"/>
-      <c r="T32" s="78" t="n"/>
+      <c r="U32" s="85" t="n"/>
+      <c r="V32" s="86" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="60" t="n"/>
-      <c r="C33" s="154" t="inlineStr">
+      <c r="B33" s="66" t="n"/>
+      <c r="C33" s="168" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="D33" s="155" t="inlineStr">
+      <c r="D33" s="169" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
-      <c r="E33" s="63" t="n"/>
-      <c r="F33" s="64" t="n"/>
-      <c r="G33" s="81" t="n"/>
-      <c r="H33" s="82" t="n"/>
-      <c r="I33" s="67" t="n"/>
-      <c r="J33" s="68" t="n"/>
-      <c r="K33" s="69" t="n"/>
-      <c r="L33" s="70" t="n"/>
-      <c r="M33" s="71" t="n"/>
-      <c r="N33" s="72" t="n"/>
-      <c r="O33" s="73" t="inlineStr">
+      <c r="E33" s="69" t="n"/>
+      <c r="F33" s="70" t="n"/>
+      <c r="G33" s="71" t="n"/>
+      <c r="H33" s="72" t="n"/>
+      <c r="I33" s="89" t="n"/>
+      <c r="J33" s="90" t="n"/>
+      <c r="K33" s="75" t="n"/>
+      <c r="L33" s="76" t="n"/>
+      <c r="M33" s="77" t="n"/>
+      <c r="N33" s="78" t="n"/>
+      <c r="O33" s="79" t="n"/>
+      <c r="P33" s="80" t="n"/>
+      <c r="Q33" s="81" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="P33" s="74" t="inlineStr">
+      <c r="R33" s="82" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
-      <c r="Q33" s="75" t="inlineStr">
+      <c r="S33" s="83" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="R33" s="76" t="inlineStr">
+      <c r="T33" s="84" t="inlineStr">
         <is>
           <t>63</t>
         </is>
       </c>
-      <c r="S33" s="77" t="n"/>
-      <c r="T33" s="78" t="n"/>
+      <c r="U33" s="85" t="n"/>
+      <c r="V33" s="86" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="60" t="n"/>
-      <c r="C34" s="154" t="inlineStr">
-        <is>
-          <t>Coin hold</t>
-        </is>
-      </c>
-      <c r="D34" s="155" t="inlineStr">
+      <c r="B34" s="66" t="n"/>
+      <c r="C34" s="168" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D34" s="169" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E34" s="63" t="n"/>
-      <c r="F34" s="64" t="n"/>
-      <c r="G34" s="81" t="n"/>
-      <c r="H34" s="82" t="n"/>
-      <c r="I34" s="67" t="n"/>
-      <c r="J34" s="68" t="n"/>
-      <c r="K34" s="69" t="n"/>
-      <c r="L34" s="70" t="n"/>
-      <c r="M34" s="71" t="n"/>
-      <c r="N34" s="72" t="n"/>
-      <c r="O34" s="73" t="inlineStr">
-        <is>
-          <t>Coin hold</t>
-        </is>
-      </c>
-      <c r="P34" s="74" t="inlineStr">
+      <c r="E34" s="170" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="Q34" s="75" t="inlineStr">
-        <is>
-          <t>Coin hold</t>
-        </is>
-      </c>
-      <c r="R34" s="76" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="S34" s="77" t="n"/>
-      <c r="T34" s="78" t="n"/>
+      <c r="F34" s="171" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G34" s="71" t="n"/>
+      <c r="H34" s="72" t="n"/>
+      <c r="I34" s="89" t="n"/>
+      <c r="J34" s="90" t="n"/>
+      <c r="K34" s="75" t="n"/>
+      <c r="L34" s="76" t="n"/>
+      <c r="M34" s="77" t="n"/>
+      <c r="N34" s="78" t="n"/>
+      <c r="O34" s="79" t="n"/>
+      <c r="P34" s="80" t="n"/>
+      <c r="Q34" s="93" t="n"/>
+      <c r="R34" s="94" t="n"/>
+      <c r="S34" s="95" t="n"/>
+      <c r="T34" s="96" t="n"/>
+      <c r="U34" s="85" t="n"/>
+      <c r="V34" s="86" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="91" t="n"/>
-      <c r="C35" s="92" t="n"/>
-      <c r="D35" s="93" t="n"/>
-      <c r="E35" s="156" t="inlineStr">
+      <c r="B35" s="99" t="n"/>
+      <c r="C35" s="100" t="n"/>
+      <c r="D35" s="101" t="n"/>
+      <c r="E35" s="102" t="n"/>
+      <c r="F35" s="103" t="n"/>
+      <c r="G35" s="172" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="F35" s="157" t="inlineStr">
+      <c r="H35" s="173" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="G35" s="158" t="inlineStr">
+      <c r="I35" s="174" t="inlineStr">
         <is>
           <t>500</t>
         </is>
       </c>
-      <c r="H35" s="159" t="inlineStr">
+      <c r="J35" s="175" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="I35" s="160" t="n"/>
-      <c r="J35" s="161" t="n"/>
-      <c r="K35" s="100" t="n"/>
-      <c r="L35" s="101" t="n"/>
-      <c r="M35" s="102" t="n"/>
-      <c r="N35" s="103" t="n"/>
-      <c r="O35" s="162" t="n"/>
-      <c r="P35" s="163" t="n"/>
-      <c r="Q35" s="164" t="n"/>
-      <c r="R35" s="165" t="n"/>
-      <c r="S35" s="108" t="n"/>
-      <c r="T35" s="109" t="n"/>
+      <c r="K35" s="176" t="n"/>
+      <c r="L35" s="177" t="n"/>
+      <c r="M35" s="110" t="n"/>
+      <c r="N35" s="111" t="n"/>
+      <c r="O35" s="112" t="n"/>
+      <c r="P35" s="113" t="n"/>
+      <c r="Q35" s="178" t="n"/>
+      <c r="R35" s="179" t="n"/>
+      <c r="S35" s="180" t="n"/>
+      <c r="T35" s="181" t="n"/>
+      <c r="U35" s="118" t="n"/>
+      <c r="V35" s="119" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="110" t="inlineStr">
+      <c r="B36" s="120" t="inlineStr">
         <is>
           <t>sum</t>
         </is>
       </c>
-      <c r="C36" s="111" t="n">
+      <c r="C36" s="121" t="n">
         <v>0</v>
       </c>
-      <c r="D36" s="112" t="n"/>
-      <c r="E36" s="113" t="n">
+      <c r="D36" s="122" t="n"/>
+      <c r="E36" s="123" t="n">
+        <v>7</v>
+      </c>
+      <c r="F36" s="124" t="n"/>
+      <c r="G36" s="125" t="n">
         <v>15595.12</v>
       </c>
-      <c r="F36" s="114" t="n"/>
-      <c r="G36" s="115" t="n">
+      <c r="H36" s="126" t="n"/>
+      <c r="I36" s="127" t="n">
         <v>541</v>
       </c>
-      <c r="H36" s="116" t="n"/>
-      <c r="I36" s="117" t="n">
+      <c r="J36" s="128" t="n"/>
+      <c r="K36" s="129" t="n">
         <v>0</v>
       </c>
-      <c r="J36" s="118" t="n"/>
-      <c r="K36" s="119" t="n">
+      <c r="L36" s="130" t="n"/>
+      <c r="M36" s="131" t="n">
         <v>0</v>
       </c>
-      <c r="L36" s="120" t="n"/>
-      <c r="M36" s="121" t="n">
+      <c r="N36" s="132" t="n"/>
+      <c r="O36" s="133" t="n">
         <v>0</v>
       </c>
-      <c r="N36" s="122" t="n"/>
-      <c r="O36" s="123" t="n">
+      <c r="P36" s="134" t="n"/>
+      <c r="Q36" s="135" t="n">
         <v>0</v>
       </c>
-      <c r="P36" s="124" t="n">
-        <v>2953.1</v>
-      </c>
-      <c r="Q36" s="125" t="n">
+      <c r="R36" s="136" t="n">
+        <v>2946.1</v>
+      </c>
+      <c r="S36" s="137" t="n">
         <v>7000</v>
       </c>
-      <c r="R36" s="126" t="n">
-        <v>5946.1</v>
-      </c>
-      <c r="S36" s="127" t="n">
-        <v>16136.12</v>
-      </c>
-      <c r="T36" s="128" t="inlineStr">
+      <c r="T36" s="138" t="n">
+        <v>5939.1</v>
+      </c>
+      <c r="U36" s="139" t="n">
+        <v>16143.12</v>
+      </c>
+      <c r="V36" s="140" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="129" t="inlineStr">
+      <c r="B37" s="141" t="inlineStr">
         <is>
           <t>total</t>
         </is>
       </c>
-      <c r="C37" s="130" t="n"/>
-      <c r="D37" s="131" t="n"/>
-      <c r="E37" s="132" t="n"/>
-      <c r="F37" s="133" t="n"/>
-      <c r="G37" s="134" t="n"/>
-      <c r="H37" s="135" t="n"/>
-      <c r="I37" s="136" t="n"/>
-      <c r="J37" s="137" t="n"/>
-      <c r="K37" s="138" t="n"/>
-      <c r="L37" s="139" t="n"/>
-      <c r="M37" s="140" t="n"/>
-      <c r="N37" s="141" t="n"/>
-      <c r="O37" s="142" t="n">
+      <c r="C37" s="142" t="n"/>
+      <c r="D37" s="143" t="n"/>
+      <c r="E37" s="144" t="n"/>
+      <c r="F37" s="145" t="n"/>
+      <c r="G37" s="146" t="n"/>
+      <c r="H37" s="147" t="n"/>
+      <c r="I37" s="148" t="n"/>
+      <c r="J37" s="149" t="n"/>
+      <c r="K37" s="150" t="n"/>
+      <c r="L37" s="151" t="n"/>
+      <c r="M37" s="152" t="n"/>
+      <c r="N37" s="153" t="n"/>
+      <c r="O37" s="154" t="n"/>
+      <c r="P37" s="155" t="n"/>
+      <c r="Q37" s="156" t="n">
         <v>0</v>
       </c>
-      <c r="P37" s="143" t="n">
-        <v>3296.8</v>
-      </c>
-      <c r="Q37" s="144" t="n">
+      <c r="R37" s="157" t="n">
+        <v>3289.8</v>
+      </c>
+      <c r="S37" s="158" t="n">
         <v>7000</v>
       </c>
-      <c r="R37" s="145" t="n">
-        <v>6289.8</v>
-      </c>
-      <c r="S37" s="146" t="n"/>
-      <c r="T37" s="147" t="n"/>
+      <c r="T37" s="159" t="n">
+        <v>6282.8</v>
+      </c>
+      <c r="U37" s="160" t="n"/>
+      <c r="V37" s="161" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="1" t="inlineStr">
@@ -2443,73 +2553,76 @@
           <t>current have</t>
         </is>
       </c>
-      <c r="C38" s="13" t="n">
+      <c r="C38" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="14" t="inlineStr">
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="E38" s="15" t="n">
-        <v>15595.12</v>
-      </c>
-      <c r="F38" s="16" t="inlineStr">
+      <c r="E38" s="182" t="n"/>
+      <c r="F38" s="35" t="n"/>
+      <c r="G38" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H38" s="19" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I38" s="20" t="n">
+        <v>541</v>
+      </c>
+      <c r="J38" s="21" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="G38" s="17" t="n">
-        <v>541</v>
-      </c>
-      <c r="H38" s="18" t="inlineStr">
+      <c r="K38" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="23" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="I38" s="19" t="n">
+      <c r="M38" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="J38" s="20" t="inlineStr">
+      <c r="N38" s="25" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="K38" s="21" t="n">
+      <c r="O38" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="L38" s="22" t="inlineStr">
+      <c r="P38" s="27" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="M38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="O38" s="37" t="n"/>
-      <c r="P38" s="38" t="n"/>
-      <c r="Q38" s="39" t="n"/>
-      <c r="R38" s="40" t="n"/>
-      <c r="S38" s="29" t="n">
-        <v>16136.12</v>
-      </c>
-      <c r="T38" s="30" t="n"/>
+      <c r="Q38" s="41" t="n"/>
+      <c r="R38" s="42" t="n"/>
+      <c r="S38" s="43" t="n"/>
+      <c r="T38" s="44" t="n"/>
+      <c r="U38" s="32" t="n">
+        <v>10541</v>
+      </c>
+      <c r="V38" s="33" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="O2:P2"/>
     <mergeCell ref="M2:N2"/>
+    <mergeCell ref="Q2:R2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="S2:U2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>